<commit_message>
Enhance ochistka.py with logging, error handling, and improved data processing
Co-authored-by: Copilot <copilot@github.com>
</commit_message>
<xml_diff>
--- a/відомість_результат.xlsx
+++ b/відомість_результат.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://robidus-my.sharepoint.com/personal/harry_boskamp_robidus_nl/Documents/Digidrat/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="11_1C7D489E14748B2492F36A925F5ED87656CF29A7" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4A9E2A1F-3ECB-45E8-A474-C73C3AE66F4C}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_37658B8E14240216F2B069925F5ED87656CF5FF8" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BDC9D6FE-1F04-4272-B7EF-3C2D05058855}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="672" uniqueCount="246">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="559" uniqueCount="244">
   <si>
     <t>Умови формування звiту</t>
   </si>
@@ -658,91 +658,85 @@
     <t>на заставі встановлено ознаку "Виключити із розрахунку КР" - "Так"</t>
   </si>
   <si>
-    <t>444078666</t>
-  </si>
-  <si>
-    <t>2521578252.UAH</t>
+    <t>DHO-104004-UAH-2404-02</t>
+  </si>
+  <si>
+    <t>N6399</t>
+  </si>
+  <si>
+    <t>Секції K,L,M,N</t>
+  </si>
+  <si>
+    <t>Прив. пiдпр.</t>
+  </si>
+  <si>
+    <t>ПАТ "Розочка"</t>
+  </si>
+  <si>
+    <t>1151214.UAH</t>
+  </si>
+  <si>
+    <t xml:space="preserve">669_62, </t>
+  </si>
+  <si>
+    <t>669_62, 662_9</t>
+  </si>
+  <si>
+    <t>DHO-104004-UAH-2404-01(2)</t>
+  </si>
+  <si>
+    <t>1151715.UAH</t>
+  </si>
+  <si>
+    <t>КІЕ-Ав-20332_240.1</t>
+  </si>
+  <si>
+    <t>N1940</t>
+  </si>
+  <si>
+    <t>АТ "Камінець-гарний"</t>
+  </si>
+  <si>
+    <t>45515555552741.UAH.555</t>
+  </si>
+  <si>
+    <t>КІЕ-Ав-20332_228.1</t>
+  </si>
+  <si>
+    <t>45517555552715.UAH.555</t>
+  </si>
+  <si>
+    <t>DNII447604674</t>
+  </si>
+  <si>
+    <t>USD</t>
+  </si>
+  <si>
+    <t>N3819</t>
+  </si>
+  <si>
+    <t>ТОВ "Рибкалов"</t>
+  </si>
+  <si>
+    <t>41222742.USD</t>
+  </si>
+  <si>
+    <t>РУШ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22, 62, </t>
+  </si>
+  <si>
+    <t>62</t>
+  </si>
+  <si>
+    <t>DNII443444421</t>
+  </si>
+  <si>
+    <t>41221752.USD</t>
   </si>
   <si>
     <t>на типі застави встановлено "Бере участь в розрахунку кредитного ризику" – «Ні»</t>
-  </si>
-  <si>
-    <t>DHO-104004-UAH-2404-02</t>
-  </si>
-  <si>
-    <t>N6399</t>
-  </si>
-  <si>
-    <t>Секції K,L,M,N</t>
-  </si>
-  <si>
-    <t>Прив. пiдпр.</t>
-  </si>
-  <si>
-    <t>ПАТ "Розочка"</t>
-  </si>
-  <si>
-    <t>1151214.UAH</t>
-  </si>
-  <si>
-    <t xml:space="preserve">669_62, </t>
-  </si>
-  <si>
-    <t>669_62, 662_9</t>
-  </si>
-  <si>
-    <t>DHO-104004-UAH-2404-01(2)</t>
-  </si>
-  <si>
-    <t>1151715.UAH</t>
-  </si>
-  <si>
-    <t>КІЕ-Ав-20332_240.1</t>
-  </si>
-  <si>
-    <t>N1940</t>
-  </si>
-  <si>
-    <t>АТ "Камінець-гарний"</t>
-  </si>
-  <si>
-    <t>45515555552741.UAH.555</t>
-  </si>
-  <si>
-    <t>КІЕ-Ав-20332_228.1</t>
-  </si>
-  <si>
-    <t>45517555552715.UAH.555</t>
-  </si>
-  <si>
-    <t>DNII447604674</t>
-  </si>
-  <si>
-    <t>USD</t>
-  </si>
-  <si>
-    <t>N3819</t>
-  </si>
-  <si>
-    <t>ТОВ "Рибкалов"</t>
-  </si>
-  <si>
-    <t>41222742.USD</t>
-  </si>
-  <si>
-    <t>РУШ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">22, 62, </t>
-  </si>
-  <si>
-    <t>62</t>
-  </si>
-  <si>
-    <t>DNII443444421</t>
-  </si>
-  <si>
-    <t>41221752.USD</t>
   </si>
   <si>
     <t>DNII443168267</t>
@@ -1101,11 +1095,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:EO40"/>
+  <dimension ref="A1:EO30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="8" max="8" width="11.7109375" customWidth="1"/>
-    <col min="9" max="9" width="17.140625" customWidth="1"/>
+    <col min="5" max="5" width="16.42578125" customWidth="1"/>
+    <col min="8" max="8" width="11.85546875" customWidth="1"/>
+    <col min="9" max="9" width="13.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:145" x14ac:dyDescent="0.25">
@@ -3547,25 +3542,25 @@
     </row>
     <row r="20" spans="1:143" x14ac:dyDescent="0.25">
       <c r="A20">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B20" t="s">
         <v>212</v>
       </c>
       <c r="C20">
-        <v>81007188</v>
+        <v>4814314</v>
       </c>
       <c r="D20">
-        <v>5000</v>
+        <v>7150</v>
       </c>
       <c r="E20" t="s">
         <v>159</v>
       </c>
       <c r="H20" s="1">
-        <v>45768</v>
+        <v>40648</v>
       </c>
       <c r="I20" s="1">
-        <v>46022</v>
+        <v>40908</v>
       </c>
       <c r="J20" t="s">
         <v>160</v>
@@ -3574,31 +3569,31 @@
         <v>1000091</v>
       </c>
       <c r="L20">
-        <v>971779</v>
+        <v>814894</v>
       </c>
       <c r="M20">
-        <v>971779</v>
+        <v>814894</v>
       </c>
       <c r="N20">
         <v>2</v>
       </c>
       <c r="O20" t="s">
-        <v>202</v>
+        <v>213</v>
       </c>
       <c r="P20" t="s">
-        <v>203</v>
+        <v>214</v>
       </c>
       <c r="Q20">
         <v>804</v>
       </c>
       <c r="R20" t="s">
-        <v>163</v>
+        <v>215</v>
       </c>
       <c r="S20">
-        <v>44112081</v>
+        <v>15918889</v>
       </c>
       <c r="T20" t="s">
-        <v>210</v>
+        <v>216</v>
       </c>
       <c r="U20" t="s">
         <v>165</v>
@@ -3610,22 +3605,16 @@
         <v>0</v>
       </c>
       <c r="Z20">
-        <v>54.8</v>
+        <v>0</v>
       </c>
       <c r="AA20" t="s">
         <v>167</v>
       </c>
       <c r="AB20">
-        <v>224</v>
-      </c>
-      <c r="AD20" t="s">
-        <v>168</v>
-      </c>
-      <c r="AE20" t="s">
-        <v>169</v>
+        <v>142</v>
       </c>
       <c r="AF20" t="s">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="AG20">
         <v>0</v>
@@ -3634,17 +3623,17 @@
         <v>0</v>
       </c>
       <c r="AK20">
-        <v>68</v>
+        <v>9</v>
       </c>
       <c r="AL20">
-        <v>68</v>
+        <v>9</v>
       </c>
       <c r="AM20" s="1"/>
       <c r="AN20">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AO20">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AP20" t="s">
         <v>171</v>
@@ -3653,19 +3642,7 @@
         <v>171</v>
       </c>
       <c r="AW20" t="s">
-        <v>165</v>
-      </c>
-      <c r="AX20">
-        <v>629776</v>
-      </c>
-      <c r="AY20" t="s">
-        <v>206</v>
-      </c>
-      <c r="AZ20">
-        <v>7</v>
-      </c>
-      <c r="BA20">
-        <v>7</v>
+        <v>171</v>
       </c>
       <c r="BB20" t="s">
         <v>171</v>
@@ -3681,7 +3658,7 @@
       </c>
       <c r="BF20" s="1"/>
       <c r="BG20" t="s">
-        <v>207</v>
+        <v>218</v>
       </c>
       <c r="BH20" t="s">
         <v>172</v>
@@ -3693,7 +3670,7 @@
         <v>171</v>
       </c>
       <c r="BN20" t="s">
-        <v>208</v>
+        <v>219</v>
       </c>
       <c r="BO20">
         <v>62</v>
@@ -3704,44 +3681,8 @@
       <c r="BT20">
         <v>6</v>
       </c>
-      <c r="BX20">
-        <v>786286878</v>
-      </c>
-      <c r="BY20">
-        <v>97927228</v>
-      </c>
-      <c r="BZ20">
-        <v>96</v>
-      </c>
-      <c r="CA20" t="s">
-        <v>182</v>
-      </c>
       <c r="CB20" s="1"/>
       <c r="CC20" s="1"/>
-      <c r="CD20" t="s">
-        <v>183</v>
-      </c>
-      <c r="CE20">
-        <v>29682</v>
-      </c>
-      <c r="CF20">
-        <v>29682</v>
-      </c>
-      <c r="CG20">
-        <v>2.276672</v>
-      </c>
-      <c r="CH20">
-        <v>2666.26</v>
-      </c>
-      <c r="CI20">
-        <v>2.9</v>
-      </c>
-      <c r="CJ20">
-        <v>2</v>
-      </c>
-      <c r="CK20">
-        <v>2</v>
-      </c>
       <c r="CL20" t="s">
         <v>171</v>
       </c>
@@ -3753,38 +3694,26 @@
       </c>
       <c r="CO20" s="1"/>
       <c r="CP20" s="1"/>
-      <c r="CS20" t="s">
-        <v>165</v>
-      </c>
-      <c r="CT20" t="s">
-        <v>209</v>
-      </c>
       <c r="CV20">
         <v>2</v>
       </c>
       <c r="CW20">
-        <v>72798922.989999995</v>
+        <v>669222</v>
       </c>
       <c r="CX20">
-        <v>72798922.989999995</v>
+        <v>669222</v>
       </c>
       <c r="CY20">
-        <v>72222222</v>
+        <v>669222</v>
       </c>
       <c r="CZ20">
-        <v>72222222</v>
-      </c>
-      <c r="DC20">
-        <v>798922.99</v>
-      </c>
-      <c r="DD20">
-        <v>798922.99</v>
+        <v>669222</v>
       </c>
       <c r="DW20">
-        <v>72798922.989999995</v>
+        <v>669222</v>
       </c>
       <c r="DX20">
-        <v>72798922.989999995</v>
+        <v>669222</v>
       </c>
       <c r="DY20">
         <v>2</v>
@@ -3793,31 +3722,22 @@
         <v>2</v>
       </c>
       <c r="EA20">
-        <v>72798922.989999995</v>
+        <v>669222</v>
       </c>
       <c r="EB20">
-        <v>72798922.989999995</v>
-      </c>
-      <c r="EC20">
-        <v>696762.78</v>
-      </c>
-      <c r="ED20">
-        <v>696762.78</v>
+        <v>669222</v>
       </c>
       <c r="EG20">
-        <v>696762.78</v>
+        <v>2</v>
       </c>
       <c r="EH20">
-        <v>696762.78</v>
-      </c>
-      <c r="EI20" t="s">
-        <v>173</v>
+        <v>2</v>
       </c>
       <c r="EJ20">
-        <v>76727699.859999999</v>
+        <v>669222</v>
       </c>
       <c r="EK20">
-        <v>76727699.859999999</v>
+        <v>669222</v>
       </c>
       <c r="EL20" t="s">
         <v>174</v>
@@ -3825,75 +3745,148 @@
       <c r="EM20" s="1"/>
     </row>
     <row r="21" spans="1:143" x14ac:dyDescent="0.25">
+      <c r="A21">
+        <v>14</v>
+      </c>
+      <c r="B21" t="s">
+        <v>220</v>
+      </c>
       <c r="C21">
-        <v>81007188</v>
+        <v>4811010</v>
       </c>
       <c r="D21">
-        <v>5000</v>
+        <v>7150</v>
       </c>
       <c r="E21" t="s">
         <v>159</v>
       </c>
-      <c r="H21" s="1"/>
-      <c r="I21" s="1"/>
+      <c r="H21" s="1">
+        <v>37068</v>
+      </c>
+      <c r="I21" s="1">
+        <v>40908</v>
+      </c>
+      <c r="J21" t="s">
+        <v>160</v>
+      </c>
+      <c r="K21">
+        <v>1000091</v>
+      </c>
       <c r="L21">
-        <v>971779</v>
+        <v>814894</v>
       </c>
       <c r="M21">
-        <v>971779</v>
+        <v>814894</v>
       </c>
       <c r="N21">
         <v>2</v>
       </c>
       <c r="O21" t="s">
-        <v>202</v>
+        <v>213</v>
+      </c>
+      <c r="P21" t="s">
+        <v>214</v>
+      </c>
+      <c r="Q21">
+        <v>804</v>
+      </c>
+      <c r="R21" t="s">
+        <v>215</v>
       </c>
       <c r="S21">
-        <v>44112081</v>
+        <v>15918889</v>
       </c>
       <c r="T21" t="s">
-        <v>210</v>
+        <v>216</v>
+      </c>
+      <c r="U21" t="s">
+        <v>165</v>
+      </c>
+      <c r="W21" t="s">
+        <v>166</v>
+      </c>
+      <c r="Y21">
+        <v>0</v>
+      </c>
+      <c r="Z21">
+        <v>0</v>
+      </c>
+      <c r="AA21" t="s">
+        <v>167</v>
+      </c>
+      <c r="AB21">
+        <v>142</v>
+      </c>
+      <c r="AF21" t="s">
+        <v>221</v>
+      </c>
+      <c r="AG21">
+        <v>0</v>
+      </c>
+      <c r="AH21">
+        <v>0</v>
+      </c>
+      <c r="AK21">
+        <v>9</v>
+      </c>
+      <c r="AL21">
+        <v>9</v>
       </c>
       <c r="AM21" s="1"/>
+      <c r="AN21">
+        <v>8</v>
+      </c>
+      <c r="AO21">
+        <v>8</v>
+      </c>
+      <c r="AP21" t="s">
+        <v>171</v>
+      </c>
+      <c r="AQ21" t="s">
+        <v>171</v>
+      </c>
+      <c r="AW21" t="s">
+        <v>171</v>
+      </c>
+      <c r="BB21" t="s">
+        <v>171</v>
+      </c>
+      <c r="BC21" t="s">
+        <v>165</v>
+      </c>
+      <c r="BD21" t="s">
+        <v>165</v>
+      </c>
+      <c r="BE21">
+        <v>6</v>
+      </c>
       <c r="BF21" s="1"/>
-      <c r="BX21">
-        <v>726968268</v>
-      </c>
-      <c r="BY21">
-        <v>79976772</v>
-      </c>
-      <c r="BZ21">
-        <v>77</v>
-      </c>
-      <c r="CA21" t="s">
-        <v>182</v>
+      <c r="BG21" t="s">
+        <v>218</v>
+      </c>
+      <c r="BH21" t="s">
+        <v>172</v>
+      </c>
+      <c r="BI21">
+        <v>69</v>
+      </c>
+      <c r="BM21" t="s">
+        <v>171</v>
+      </c>
+      <c r="BN21" t="s">
+        <v>219</v>
+      </c>
+      <c r="BO21">
+        <v>62</v>
+      </c>
+      <c r="BS21">
+        <v>62</v>
+      </c>
+      <c r="BT21">
+        <v>6</v>
       </c>
       <c r="CB21" s="1"/>
       <c r="CC21" s="1"/>
-      <c r="CD21" t="s">
-        <v>174</v>
-      </c>
-      <c r="CE21">
-        <v>827222779.70000005</v>
-      </c>
-      <c r="CF21">
-        <v>827222779.70000005</v>
-      </c>
-      <c r="CG21">
-        <v>2.2798289999999999</v>
-      </c>
-      <c r="CH21">
-        <v>72798922.959999993</v>
-      </c>
-      <c r="CI21">
-        <v>2.8</v>
-      </c>
-      <c r="CJ21">
-        <v>2</v>
-      </c>
-      <c r="CK21">
-        <v>2</v>
-      </c>
       <c r="CL21" t="s">
         <v>171</v>
       </c>
@@ -3905,60 +3898,184 @@
       </c>
       <c r="CO21" s="1"/>
       <c r="CP21" s="1"/>
-      <c r="CS21" t="s">
-        <v>165</v>
-      </c>
-      <c r="CT21" t="s">
-        <v>214</v>
+      <c r="CV21">
+        <v>2</v>
+      </c>
+      <c r="CW21">
+        <v>7672222</v>
+      </c>
+      <c r="CX21">
+        <v>7672222</v>
+      </c>
+      <c r="CY21">
+        <v>7672222</v>
+      </c>
+      <c r="CZ21">
+        <v>7672222</v>
+      </c>
+      <c r="DW21">
+        <v>7672222</v>
+      </c>
+      <c r="DX21">
+        <v>7672222</v>
+      </c>
+      <c r="DY21">
+        <v>2</v>
+      </c>
+      <c r="DZ21">
+        <v>2</v>
+      </c>
+      <c r="EA21">
+        <v>7672222</v>
+      </c>
+      <c r="EB21">
+        <v>7672222</v>
+      </c>
+      <c r="EG21">
+        <v>2</v>
+      </c>
+      <c r="EH21">
+        <v>2</v>
       </c>
       <c r="EJ21">
-        <v>2</v>
+        <v>7672222</v>
       </c>
       <c r="EK21">
-        <v>2</v>
+        <v>7672222</v>
+      </c>
+      <c r="EL21" t="s">
+        <v>174</v>
       </c>
       <c r="EM21" s="1"/>
     </row>
     <row r="22" spans="1:143" x14ac:dyDescent="0.25">
+      <c r="A22">
+        <v>15</v>
+      </c>
+      <c r="B22" t="s">
+        <v>222</v>
+      </c>
       <c r="C22">
-        <v>81007188</v>
+        <v>104111348</v>
       </c>
       <c r="D22">
-        <v>5000</v>
+        <v>7160</v>
       </c>
       <c r="E22" t="s">
-        <v>159</v>
-      </c>
-      <c r="H22" s="1"/>
-      <c r="I22" s="1"/>
+        <v>176</v>
+      </c>
+      <c r="H22" s="1">
+        <v>45965</v>
+      </c>
+      <c r="I22" s="1">
+        <v>46057</v>
+      </c>
+      <c r="J22" t="s">
+        <v>160</v>
+      </c>
+      <c r="K22">
+        <v>1000091</v>
+      </c>
       <c r="L22">
-        <v>971779</v>
+        <v>811681</v>
       </c>
       <c r="M22">
-        <v>971779</v>
+        <v>811681</v>
       </c>
       <c r="N22">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O22" t="s">
-        <v>202</v>
+        <v>223</v>
+      </c>
+      <c r="Q22">
+        <v>804</v>
+      </c>
+      <c r="R22" t="s">
+        <v>163</v>
       </c>
       <c r="S22">
-        <v>44112081</v>
+        <v>154108</v>
       </c>
       <c r="T22" t="s">
-        <v>210</v>
+        <v>224</v>
+      </c>
+      <c r="U22" t="s">
+        <v>165</v>
+      </c>
+      <c r="W22" t="s">
+        <v>166</v>
+      </c>
+      <c r="Y22">
+        <v>0</v>
+      </c>
+      <c r="AA22" t="s">
+        <v>167</v>
+      </c>
+      <c r="AB22">
+        <v>182</v>
+      </c>
+      <c r="AF22" t="s">
+        <v>225</v>
+      </c>
+      <c r="AG22">
+        <v>0</v>
+      </c>
+      <c r="AH22">
+        <v>0</v>
+      </c>
+      <c r="AK22">
+        <v>9</v>
+      </c>
+      <c r="AL22">
+        <v>9</v>
       </c>
       <c r="AM22" s="1"/>
+      <c r="AO22">
+        <v>9</v>
+      </c>
+      <c r="AP22" t="s">
+        <v>171</v>
+      </c>
+      <c r="AQ22" t="s">
+        <v>171</v>
+      </c>
+      <c r="AW22" t="s">
+        <v>171</v>
+      </c>
+      <c r="BB22" t="s">
+        <v>171</v>
+      </c>
+      <c r="BC22" t="s">
+        <v>171</v>
+      </c>
+      <c r="BD22" t="s">
+        <v>171</v>
+      </c>
       <c r="BF22" s="1"/>
-      <c r="BX22">
-        <v>786282629</v>
+      <c r="BH22" t="s">
+        <v>172</v>
+      </c>
+      <c r="BJ22">
+        <v>9</v>
+      </c>
+      <c r="BM22" t="s">
+        <v>171</v>
+      </c>
+      <c r="BP22">
+        <v>9</v>
+      </c>
+      <c r="BS22">
+        <v>9</v>
+      </c>
+      <c r="BV22">
+        <v>6</v>
       </c>
       <c r="BY22">
-        <v>97927897</v>
+        <v>69989976</v>
       </c>
       <c r="BZ22">
-        <v>96</v>
+        <v>76</v>
       </c>
       <c r="CA22" t="s">
         <v>182</v>
@@ -3969,20 +4086,20 @@
         <v>183</v>
       </c>
       <c r="CE22">
+        <v>2</v>
+      </c>
+      <c r="CF22">
+        <v>2</v>
+      </c>
+      <c r="CG22">
         <v>6</v>
       </c>
-      <c r="CF22">
+      <c r="CH22">
+        <v>2</v>
+      </c>
+      <c r="CI22">
         <v>6</v>
       </c>
-      <c r="CG22">
-        <v>2.276672</v>
-      </c>
-      <c r="CH22">
-        <v>2.27</v>
-      </c>
-      <c r="CI22">
-        <v>2.9</v>
-      </c>
       <c r="CJ22">
         <v>2</v>
       </c>
@@ -3996,64 +4113,191 @@
         <v>171</v>
       </c>
       <c r="CN22">
-        <v>2</v>
+        <v>92.29</v>
       </c>
       <c r="CO22" s="1"/>
       <c r="CP22" s="1"/>
       <c r="CS22" t="s">
-        <v>165</v>
-      </c>
-      <c r="CT22" t="s">
-        <v>211</v>
+        <v>171</v>
+      </c>
+      <c r="CV22">
+        <v>2</v>
+      </c>
+      <c r="DO22">
+        <v>87766829.989999995</v>
+      </c>
+      <c r="DP22">
+        <v>87766829.989999995</v>
+      </c>
+      <c r="DQ22">
+        <v>87727287.680000007</v>
+      </c>
+      <c r="DR22">
+        <v>87727287.680000007</v>
+      </c>
+      <c r="DS22">
+        <v>87766.86</v>
+      </c>
+      <c r="DT22">
+        <v>87766.86</v>
+      </c>
+      <c r="DY22">
+        <v>2</v>
+      </c>
+      <c r="DZ22">
+        <v>2</v>
+      </c>
+      <c r="EA22">
+        <v>2</v>
+      </c>
+      <c r="EB22">
+        <v>2</v>
+      </c>
+      <c r="EG22">
+        <v>2</v>
+      </c>
+      <c r="EH22">
+        <v>2</v>
       </c>
       <c r="EJ22">
         <v>2</v>
       </c>
       <c r="EK22">
         <v>2</v>
+      </c>
+      <c r="EL22" t="s">
+        <v>174</v>
       </c>
       <c r="EM22" s="1"/>
     </row>
     <row r="23" spans="1:143" x14ac:dyDescent="0.25">
+      <c r="A23">
+        <v>16</v>
+      </c>
+      <c r="B23" t="s">
+        <v>226</v>
+      </c>
       <c r="C23">
-        <v>81007188</v>
+        <v>104414770</v>
       </c>
       <c r="D23">
-        <v>5000</v>
+        <v>7160</v>
       </c>
       <c r="E23" t="s">
-        <v>159</v>
-      </c>
-      <c r="H23" s="1"/>
-      <c r="I23" s="1"/>
+        <v>176</v>
+      </c>
+      <c r="H23" s="1">
+        <v>45965</v>
+      </c>
+      <c r="I23" s="1">
+        <v>46052</v>
+      </c>
+      <c r="J23" t="s">
+        <v>160</v>
+      </c>
+      <c r="K23">
+        <v>1000091</v>
+      </c>
       <c r="L23">
-        <v>971779</v>
+        <v>811681</v>
       </c>
       <c r="M23">
-        <v>971779</v>
+        <v>811681</v>
       </c>
       <c r="N23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O23" t="s">
-        <v>202</v>
+        <v>223</v>
+      </c>
+      <c r="Q23">
+        <v>804</v>
+      </c>
+      <c r="R23" t="s">
+        <v>163</v>
       </c>
       <c r="S23">
-        <v>44112081</v>
+        <v>154108</v>
       </c>
       <c r="T23" t="s">
-        <v>210</v>
+        <v>224</v>
+      </c>
+      <c r="U23" t="s">
+        <v>165</v>
+      </c>
+      <c r="W23" t="s">
+        <v>166</v>
+      </c>
+      <c r="Y23">
+        <v>0</v>
+      </c>
+      <c r="AA23" t="s">
+        <v>167</v>
+      </c>
+      <c r="AB23">
+        <v>182</v>
+      </c>
+      <c r="AF23" t="s">
+        <v>227</v>
+      </c>
+      <c r="AG23">
+        <v>0</v>
+      </c>
+      <c r="AH23">
+        <v>0</v>
+      </c>
+      <c r="AK23">
+        <v>9</v>
+      </c>
+      <c r="AL23">
+        <v>9</v>
       </c>
       <c r="AM23" s="1"/>
+      <c r="AO23">
+        <v>9</v>
+      </c>
+      <c r="AP23" t="s">
+        <v>171</v>
+      </c>
+      <c r="AQ23" t="s">
+        <v>171</v>
+      </c>
+      <c r="AW23" t="s">
+        <v>171</v>
+      </c>
+      <c r="BB23" t="s">
+        <v>171</v>
+      </c>
+      <c r="BC23" t="s">
+        <v>171</v>
+      </c>
+      <c r="BD23" t="s">
+        <v>171</v>
+      </c>
       <c r="BF23" s="1"/>
-      <c r="BX23">
-        <v>786286876</v>
+      <c r="BH23" t="s">
+        <v>172</v>
+      </c>
+      <c r="BJ23">
+        <v>9</v>
+      </c>
+      <c r="BM23" t="s">
+        <v>171</v>
+      </c>
+      <c r="BP23">
+        <v>9</v>
+      </c>
+      <c r="BS23">
+        <v>9</v>
+      </c>
+      <c r="BV23">
+        <v>6</v>
       </c>
       <c r="BY23">
-        <v>97927266</v>
+        <v>69989976</v>
       </c>
       <c r="BZ23">
-        <v>96</v>
+        <v>76</v>
       </c>
       <c r="CA23" t="s">
         <v>182</v>
@@ -4064,19 +4308,19 @@
         <v>183</v>
       </c>
       <c r="CE23">
-        <v>82726</v>
+        <v>2</v>
       </c>
       <c r="CF23">
-        <v>82726</v>
+        <v>2</v>
       </c>
       <c r="CG23">
-        <v>2.276672</v>
+        <v>6</v>
       </c>
       <c r="CH23">
-        <v>7228.97</v>
+        <v>2</v>
       </c>
       <c r="CI23">
-        <v>2.9</v>
+        <v>6</v>
       </c>
       <c r="CJ23">
         <v>2</v>
@@ -4091,61 +4335,230 @@
         <v>171</v>
       </c>
       <c r="CN23">
-        <v>2</v>
+        <v>92.29</v>
       </c>
       <c r="CO23" s="1"/>
       <c r="CP23" s="1"/>
       <c r="CS23" t="s">
-        <v>165</v>
-      </c>
-      <c r="CT23" t="s">
-        <v>209</v>
+        <v>171</v>
+      </c>
+      <c r="CV23">
+        <v>2</v>
+      </c>
+      <c r="DO23">
+        <v>8677286.9600000009</v>
+      </c>
+      <c r="DP23">
+        <v>8677286.9600000009</v>
+      </c>
+      <c r="DQ23">
+        <v>8668628.6699999999</v>
+      </c>
+      <c r="DR23">
+        <v>8668628.6699999999</v>
+      </c>
+      <c r="DS23">
+        <v>8677.2800000000007</v>
+      </c>
+      <c r="DT23">
+        <v>8677.2800000000007</v>
+      </c>
+      <c r="DY23">
+        <v>2</v>
+      </c>
+      <c r="DZ23">
+        <v>2</v>
+      </c>
+      <c r="EA23">
+        <v>2</v>
+      </c>
+      <c r="EB23">
+        <v>2</v>
+      </c>
+      <c r="EG23">
+        <v>2</v>
+      </c>
+      <c r="EH23">
+        <v>2</v>
       </c>
       <c r="EJ23">
         <v>2</v>
       </c>
       <c r="EK23">
         <v>2</v>
+      </c>
+      <c r="EL23" t="s">
+        <v>174</v>
       </c>
       <c r="EM23" s="1"/>
     </row>
     <row r="24" spans="1:143" x14ac:dyDescent="0.25">
+      <c r="A24">
+        <v>17</v>
+      </c>
+      <c r="B24" t="s">
+        <v>228</v>
+      </c>
       <c r="C24">
-        <v>81007188</v>
+        <v>88441027</v>
       </c>
       <c r="D24">
-        <v>5000</v>
+        <v>7003</v>
       </c>
       <c r="E24" t="s">
-        <v>159</v>
-      </c>
-      <c r="H24" s="1"/>
-      <c r="I24" s="1"/>
+        <v>176</v>
+      </c>
+      <c r="F24" t="s">
+        <v>229</v>
+      </c>
+      <c r="G24">
+        <v>42.094799999999999</v>
+      </c>
+      <c r="H24" s="1">
+        <v>45763</v>
+      </c>
+      <c r="I24" s="1">
+        <v>46024</v>
+      </c>
+      <c r="J24" t="s">
+        <v>160</v>
+      </c>
+      <c r="K24">
+        <v>1000091</v>
+      </c>
       <c r="L24">
-        <v>971779</v>
+        <v>867006</v>
       </c>
       <c r="M24">
-        <v>971779</v>
+        <v>867006</v>
       </c>
       <c r="N24">
         <v>2</v>
       </c>
       <c r="O24" t="s">
-        <v>202</v>
+        <v>230</v>
+      </c>
+      <c r="P24" t="s">
+        <v>203</v>
+      </c>
+      <c r="Q24">
+        <v>804</v>
+      </c>
+      <c r="R24" t="s">
+        <v>163</v>
       </c>
       <c r="S24">
-        <v>44112081</v>
+        <v>14008840</v>
       </c>
       <c r="T24" t="s">
-        <v>210</v>
+        <v>231</v>
+      </c>
+      <c r="U24" t="s">
+        <v>165</v>
+      </c>
+      <c r="W24" t="s">
+        <v>166</v>
+      </c>
+      <c r="Y24">
+        <v>0</v>
+      </c>
+      <c r="Z24">
+        <v>85.8</v>
+      </c>
+      <c r="AA24" t="s">
+        <v>167</v>
+      </c>
+      <c r="AB24">
+        <v>221</v>
+      </c>
+      <c r="AF24" t="s">
+        <v>232</v>
+      </c>
+      <c r="AG24">
+        <v>0</v>
+      </c>
+      <c r="AH24">
+        <v>0</v>
+      </c>
+      <c r="AI24">
+        <v>0</v>
+      </c>
+      <c r="AK24">
+        <v>8.9</v>
+      </c>
+      <c r="AL24">
+        <v>8.9</v>
       </c>
       <c r="AM24" s="1"/>
+      <c r="AN24">
+        <v>6</v>
+      </c>
+      <c r="AO24">
+        <v>2</v>
+      </c>
+      <c r="AP24" t="s">
+        <v>171</v>
+      </c>
+      <c r="AQ24" t="s">
+        <v>165</v>
+      </c>
+      <c r="AR24">
+        <v>267226</v>
+      </c>
+      <c r="AS24" t="s">
+        <v>233</v>
+      </c>
+      <c r="AT24">
+        <v>2</v>
+      </c>
+      <c r="AU24">
+        <v>2</v>
+      </c>
+      <c r="AW24" t="s">
+        <v>171</v>
+      </c>
+      <c r="BB24" t="s">
+        <v>171</v>
+      </c>
+      <c r="BC24" t="s">
+        <v>171</v>
+      </c>
+      <c r="BD24" t="s">
+        <v>171</v>
+      </c>
       <c r="BF24" s="1"/>
+      <c r="BG24" t="s">
+        <v>234</v>
+      </c>
+      <c r="BH24" t="s">
+        <v>172</v>
+      </c>
+      <c r="BJ24">
+        <v>2</v>
+      </c>
+      <c r="BM24" t="s">
+        <v>171</v>
+      </c>
+      <c r="BN24" t="s">
+        <v>235</v>
+      </c>
+      <c r="BP24">
+        <v>2</v>
+      </c>
+      <c r="BS24">
+        <v>2</v>
+      </c>
+      <c r="BT24">
+        <v>2.2698</v>
+      </c>
+      <c r="BV24">
+        <v>6</v>
+      </c>
       <c r="BX24">
-        <v>788762767</v>
+        <v>787688828</v>
       </c>
       <c r="BY24">
-        <v>622667622</v>
+        <v>98986787</v>
       </c>
       <c r="BZ24">
         <v>96</v>
@@ -4159,16 +4572,16 @@
         <v>183</v>
       </c>
       <c r="CE24">
-        <v>67688</v>
+        <v>682228</v>
       </c>
       <c r="CF24">
-        <v>67688</v>
+        <v>682228</v>
       </c>
       <c r="CG24">
-        <v>2.276672</v>
+        <v>2.2887680000000001</v>
       </c>
       <c r="CH24">
-        <v>8778.9599999999991</v>
+        <v>96879.89</v>
       </c>
       <c r="CI24">
         <v>2.9</v>
@@ -4194,53 +4607,225 @@
         <v>165</v>
       </c>
       <c r="CT24" t="s">
-        <v>209</v>
+        <v>211</v>
+      </c>
+      <c r="CV24">
+        <v>2</v>
+      </c>
+      <c r="DO24">
+        <v>927696.66</v>
+      </c>
+      <c r="DP24">
+        <v>22226962.789999999</v>
+      </c>
+      <c r="DQ24">
+        <v>927696.66</v>
+      </c>
+      <c r="DR24">
+        <v>22226962.789999999</v>
+      </c>
+      <c r="DW24">
+        <v>62689.68</v>
+      </c>
+      <c r="DX24">
+        <v>827226.22</v>
+      </c>
+      <c r="DY24">
+        <v>2</v>
+      </c>
+      <c r="DZ24">
+        <v>2</v>
+      </c>
+      <c r="EA24">
+        <v>62689.68</v>
+      </c>
+      <c r="EB24">
+        <v>827226.22</v>
+      </c>
+      <c r="EG24">
+        <v>2</v>
+      </c>
+      <c r="EH24">
+        <v>2</v>
       </c>
       <c r="EJ24">
-        <v>2</v>
+        <v>62689.68</v>
       </c>
       <c r="EK24">
-        <v>2</v>
+        <v>827226.22</v>
+      </c>
+      <c r="EL24" t="s">
+        <v>174</v>
       </c>
       <c r="EM24" s="1"/>
     </row>
     <row r="25" spans="1:143" x14ac:dyDescent="0.25">
+      <c r="A25">
+        <v>18</v>
+      </c>
+      <c r="B25" t="s">
+        <v>236</v>
+      </c>
       <c r="C25">
-        <v>81007188</v>
+        <v>100243246</v>
       </c>
       <c r="D25">
-        <v>5000</v>
+        <v>7003</v>
       </c>
       <c r="E25" t="s">
-        <v>159</v>
-      </c>
-      <c r="H25" s="1"/>
-      <c r="I25" s="1"/>
+        <v>176</v>
+      </c>
+      <c r="F25" t="s">
+        <v>229</v>
+      </c>
+      <c r="G25">
+        <v>42.094799999999999</v>
+      </c>
+      <c r="H25" s="1">
+        <v>45690</v>
+      </c>
+      <c r="I25" s="1">
+        <v>46024</v>
+      </c>
+      <c r="J25" t="s">
+        <v>160</v>
+      </c>
+      <c r="K25">
+        <v>1000091</v>
+      </c>
       <c r="L25">
-        <v>971779</v>
+        <v>867006</v>
       </c>
       <c r="M25">
-        <v>971779</v>
+        <v>867006</v>
       </c>
       <c r="N25">
         <v>2</v>
       </c>
       <c r="O25" t="s">
-        <v>202</v>
+        <v>230</v>
+      </c>
+      <c r="P25" t="s">
+        <v>203</v>
+      </c>
+      <c r="Q25">
+        <v>804</v>
+      </c>
+      <c r="R25" t="s">
+        <v>163</v>
       </c>
       <c r="S25">
-        <v>44112081</v>
+        <v>14008840</v>
       </c>
       <c r="T25" t="s">
-        <v>210</v>
+        <v>231</v>
+      </c>
+      <c r="U25" t="s">
+        <v>165</v>
+      </c>
+      <c r="W25" t="s">
+        <v>166</v>
+      </c>
+      <c r="Y25">
+        <v>0</v>
+      </c>
+      <c r="Z25">
+        <v>85.8</v>
+      </c>
+      <c r="AA25" t="s">
+        <v>167</v>
+      </c>
+      <c r="AB25">
+        <v>221</v>
+      </c>
+      <c r="AF25" t="s">
+        <v>237</v>
+      </c>
+      <c r="AG25">
+        <v>0</v>
+      </c>
+      <c r="AH25">
+        <v>0</v>
+      </c>
+      <c r="AI25">
+        <v>0</v>
+      </c>
+      <c r="AK25">
+        <v>8.9</v>
+      </c>
+      <c r="AL25">
+        <v>8.9</v>
       </c>
       <c r="AM25" s="1"/>
+      <c r="AN25">
+        <v>6</v>
+      </c>
+      <c r="AO25">
+        <v>2</v>
+      </c>
+      <c r="AP25" t="s">
+        <v>171</v>
+      </c>
+      <c r="AQ25" t="s">
+        <v>165</v>
+      </c>
+      <c r="AR25">
+        <v>267226</v>
+      </c>
+      <c r="AS25" t="s">
+        <v>233</v>
+      </c>
+      <c r="AT25">
+        <v>2</v>
+      </c>
+      <c r="AU25">
+        <v>2</v>
+      </c>
+      <c r="AW25" t="s">
+        <v>171</v>
+      </c>
+      <c r="BB25" t="s">
+        <v>171</v>
+      </c>
+      <c r="BC25" t="s">
+        <v>171</v>
+      </c>
+      <c r="BD25" t="s">
+        <v>171</v>
+      </c>
       <c r="BF25" s="1"/>
+      <c r="BG25" t="s">
+        <v>234</v>
+      </c>
+      <c r="BH25" t="s">
+        <v>172</v>
+      </c>
+      <c r="BJ25">
+        <v>2</v>
+      </c>
+      <c r="BM25" t="s">
+        <v>171</v>
+      </c>
+      <c r="BN25" t="s">
+        <v>235</v>
+      </c>
+      <c r="BP25">
+        <v>2</v>
+      </c>
+      <c r="BS25">
+        <v>2</v>
+      </c>
+      <c r="BT25">
+        <v>2.2698</v>
+      </c>
+      <c r="BV25">
+        <v>6</v>
+      </c>
       <c r="BX25">
-        <v>726966892</v>
+        <v>286979998</v>
       </c>
       <c r="BY25">
-        <v>79978686</v>
+        <v>78266622</v>
       </c>
       <c r="BZ25">
         <v>77</v>
@@ -4254,16 +4839,16 @@
         <v>174</v>
       </c>
       <c r="CE25">
-        <v>899866278.60000002</v>
+        <v>778268229.29999995</v>
       </c>
       <c r="CF25">
-        <v>899866278.60000002</v>
+        <v>778268229.29999995</v>
       </c>
       <c r="CG25">
-        <v>2.276672</v>
+        <v>2.6627890000000001</v>
       </c>
       <c r="CH25">
-        <v>72798922.980000004</v>
+        <v>228698696.90000001</v>
       </c>
       <c r="CI25">
         <v>2.8</v>
@@ -4285,57 +4870,232 @@
       </c>
       <c r="CO25" s="1"/>
       <c r="CP25" s="1"/>
+      <c r="CQ25" t="s">
+        <v>171</v>
+      </c>
       <c r="CS25" t="s">
         <v>165</v>
       </c>
       <c r="CT25" t="s">
-        <v>214</v>
+        <v>238</v>
+      </c>
+      <c r="CV25">
+        <v>2</v>
+      </c>
+      <c r="DO25">
+        <v>62686</v>
+      </c>
+      <c r="DP25">
+        <v>2676862.77</v>
+      </c>
+      <c r="DQ25">
+        <v>62686</v>
+      </c>
+      <c r="DR25">
+        <v>2676862.77</v>
+      </c>
+      <c r="DW25">
+        <v>6269.28</v>
+      </c>
+      <c r="DX25">
+        <v>96699.28</v>
+      </c>
+      <c r="DY25">
+        <v>2</v>
+      </c>
+      <c r="DZ25">
+        <v>2</v>
+      </c>
+      <c r="EA25">
+        <v>6269.28</v>
+      </c>
+      <c r="EB25">
+        <v>96699.28</v>
+      </c>
+      <c r="EG25">
+        <v>2</v>
+      </c>
+      <c r="EH25">
+        <v>2</v>
       </c>
       <c r="EJ25">
-        <v>2</v>
+        <v>6269.28</v>
       </c>
       <c r="EK25">
-        <v>2</v>
+        <v>96699.28</v>
+      </c>
+      <c r="EL25" t="s">
+        <v>174</v>
       </c>
       <c r="EM25" s="1"/>
     </row>
     <row r="26" spans="1:143" x14ac:dyDescent="0.25">
+      <c r="A26">
+        <v>19</v>
+      </c>
+      <c r="B26" t="s">
+        <v>239</v>
+      </c>
       <c r="C26">
-        <v>81007188</v>
+        <v>100461040</v>
       </c>
       <c r="D26">
-        <v>5000</v>
+        <v>7003</v>
       </c>
       <c r="E26" t="s">
-        <v>159</v>
-      </c>
-      <c r="H26" s="1"/>
-      <c r="I26" s="1"/>
+        <v>176</v>
+      </c>
+      <c r="F26" t="s">
+        <v>229</v>
+      </c>
+      <c r="G26">
+        <v>42.094799999999999</v>
+      </c>
+      <c r="H26" s="1">
+        <v>45700</v>
+      </c>
+      <c r="I26" s="1">
+        <v>46017</v>
+      </c>
+      <c r="J26" t="s">
+        <v>160</v>
+      </c>
+      <c r="K26">
+        <v>1000091</v>
+      </c>
       <c r="L26">
-        <v>971779</v>
+        <v>867006</v>
       </c>
       <c r="M26">
-        <v>971779</v>
+        <v>867006</v>
       </c>
       <c r="N26">
         <v>2</v>
       </c>
       <c r="O26" t="s">
-        <v>202</v>
+        <v>230</v>
+      </c>
+      <c r="P26" t="s">
+        <v>203</v>
+      </c>
+      <c r="Q26">
+        <v>804</v>
+      </c>
+      <c r="R26" t="s">
+        <v>163</v>
       </c>
       <c r="S26">
-        <v>44112081</v>
+        <v>14008840</v>
       </c>
       <c r="T26" t="s">
-        <v>210</v>
+        <v>231</v>
+      </c>
+      <c r="U26" t="s">
+        <v>165</v>
+      </c>
+      <c r="W26" t="s">
+        <v>166</v>
+      </c>
+      <c r="Y26">
+        <v>0</v>
+      </c>
+      <c r="Z26">
+        <v>85.8</v>
+      </c>
+      <c r="AA26" t="s">
+        <v>167</v>
+      </c>
+      <c r="AB26">
+        <v>221</v>
+      </c>
+      <c r="AF26" t="s">
+        <v>240</v>
+      </c>
+      <c r="AG26">
+        <v>0</v>
+      </c>
+      <c r="AH26">
+        <v>0</v>
+      </c>
+      <c r="AI26">
+        <v>0</v>
+      </c>
+      <c r="AK26">
+        <v>8.9</v>
+      </c>
+      <c r="AL26">
+        <v>8.9</v>
       </c>
       <c r="AM26" s="1"/>
+      <c r="AN26">
+        <v>6</v>
+      </c>
+      <c r="AO26">
+        <v>2</v>
+      </c>
+      <c r="AP26" t="s">
+        <v>171</v>
+      </c>
+      <c r="AQ26" t="s">
+        <v>165</v>
+      </c>
+      <c r="AR26">
+        <v>267226</v>
+      </c>
+      <c r="AS26" t="s">
+        <v>233</v>
+      </c>
+      <c r="AT26">
+        <v>2</v>
+      </c>
+      <c r="AU26">
+        <v>2</v>
+      </c>
+      <c r="AW26" t="s">
+        <v>171</v>
+      </c>
+      <c r="BB26" t="s">
+        <v>171</v>
+      </c>
+      <c r="BC26" t="s">
+        <v>171</v>
+      </c>
+      <c r="BD26" t="s">
+        <v>171</v>
+      </c>
       <c r="BF26" s="1"/>
+      <c r="BG26" t="s">
+        <v>234</v>
+      </c>
+      <c r="BH26" t="s">
+        <v>172</v>
+      </c>
+      <c r="BJ26">
+        <v>2</v>
+      </c>
+      <c r="BM26" t="s">
+        <v>171</v>
+      </c>
+      <c r="BN26" t="s">
+        <v>235</v>
+      </c>
+      <c r="BP26">
+        <v>2</v>
+      </c>
+      <c r="BS26">
+        <v>2</v>
+      </c>
+      <c r="BT26">
+        <v>2.2698</v>
+      </c>
+      <c r="BV26">
+        <v>6</v>
+      </c>
       <c r="BX26">
-        <v>786282677</v>
+        <v>787688798</v>
       </c>
       <c r="BY26">
-        <v>97927897</v>
+        <v>98986628</v>
       </c>
       <c r="BZ26">
         <v>96</v>
@@ -4349,16 +5109,16 @@
         <v>183</v>
       </c>
       <c r="CE26">
-        <v>69779</v>
+        <v>289866</v>
       </c>
       <c r="CF26">
-        <v>69779</v>
+        <v>289866</v>
       </c>
       <c r="CG26">
-        <v>2.276672</v>
+        <v>2.2887680000000001</v>
       </c>
       <c r="CH26">
-        <v>6778.69</v>
+        <v>76278.679999999993</v>
       </c>
       <c r="CI26">
         <v>2.9</v>
@@ -4384,2276 +5144,377 @@
         <v>165</v>
       </c>
       <c r="CT26" t="s">
-        <v>209</v>
+        <v>211</v>
+      </c>
+      <c r="CV26">
+        <v>2</v>
+      </c>
+      <c r="DO26">
+        <v>26276.79</v>
+      </c>
+      <c r="DP26">
+        <v>6299826.7599999998</v>
+      </c>
+      <c r="DQ26">
+        <v>26276.79</v>
+      </c>
+      <c r="DR26">
+        <v>6299826.7599999998</v>
+      </c>
+      <c r="DW26">
+        <v>929.22</v>
+      </c>
+      <c r="DX26">
+        <v>26298.720000000001</v>
+      </c>
+      <c r="DY26">
+        <v>2</v>
+      </c>
+      <c r="DZ26">
+        <v>2</v>
+      </c>
+      <c r="EA26">
+        <v>929.22</v>
+      </c>
+      <c r="EB26">
+        <v>26298.720000000001</v>
+      </c>
+      <c r="EG26">
+        <v>2</v>
+      </c>
+      <c r="EH26">
+        <v>2</v>
       </c>
       <c r="EJ26">
-        <v>2</v>
+        <v>929.22</v>
       </c>
       <c r="EK26">
-        <v>2</v>
+        <v>26298.720000000001</v>
+      </c>
+      <c r="EL26" t="s">
+        <v>174</v>
       </c>
       <c r="EM26" s="1"/>
     </row>
     <row r="27" spans="1:143" x14ac:dyDescent="0.25">
-      <c r="C27">
-        <v>81007188</v>
-      </c>
       <c r="D27">
-        <v>5000</v>
-      </c>
-      <c r="E27" t="s">
-        <v>159</v>
+        <v>7003</v>
+      </c>
+      <c r="F27" t="s">
+        <v>241</v>
       </c>
       <c r="H27" s="1"/>
       <c r="I27" s="1"/>
-      <c r="L27">
-        <v>971779</v>
-      </c>
-      <c r="M27">
-        <v>971779</v>
-      </c>
-      <c r="N27">
-        <v>2</v>
-      </c>
-      <c r="O27" t="s">
-        <v>202</v>
-      </c>
       <c r="S27">
-        <v>44112081</v>
-      </c>
-      <c r="T27" t="s">
-        <v>210</v>
+        <v>14008840</v>
       </c>
       <c r="AM27" s="1"/>
       <c r="BF27" s="1"/>
-      <c r="BX27">
-        <v>786286877</v>
-      </c>
-      <c r="BY27">
-        <v>97927269</v>
-      </c>
-      <c r="BZ27">
-        <v>96</v>
-      </c>
-      <c r="CA27" t="s">
-        <v>182</v>
-      </c>
       <c r="CB27" s="1"/>
       <c r="CC27" s="1"/>
-      <c r="CD27" t="s">
-        <v>183</v>
-      </c>
-      <c r="CE27">
-        <v>99888</v>
-      </c>
-      <c r="CF27">
-        <v>99888</v>
-      </c>
-      <c r="CG27">
-        <v>2.276672</v>
-      </c>
-      <c r="CH27">
-        <v>8299.98</v>
-      </c>
-      <c r="CI27">
-        <v>2.9</v>
-      </c>
-      <c r="CJ27">
-        <v>2</v>
-      </c>
-      <c r="CK27">
-        <v>2</v>
-      </c>
-      <c r="CL27" t="s">
-        <v>171</v>
-      </c>
-      <c r="CM27" t="s">
-        <v>171</v>
-      </c>
-      <c r="CN27">
-        <v>2</v>
-      </c>
       <c r="CO27" s="1"/>
       <c r="CP27" s="1"/>
-      <c r="CS27" t="s">
-        <v>165</v>
-      </c>
-      <c r="CT27" t="s">
-        <v>209</v>
+      <c r="CW27">
+        <v>99649294194</v>
+      </c>
+      <c r="CX27">
+        <v>99649294194</v>
+      </c>
+      <c r="DO27">
+        <v>41211221112</v>
+      </c>
+      <c r="DP27">
+        <v>41211221112</v>
+      </c>
+      <c r="DQ27">
+        <v>69222669996</v>
+      </c>
+      <c r="DR27">
+        <v>69222669996</v>
+      </c>
+      <c r="DS27">
+        <v>196929027</v>
+      </c>
+      <c r="DT27">
+        <v>196929027</v>
+      </c>
+      <c r="DU27">
+        <v>2161.91</v>
+      </c>
+      <c r="DV27">
+        <v>2161.91</v>
+      </c>
+      <c r="DW27">
+        <v>11920144926</v>
+      </c>
+      <c r="DX27">
+        <v>11920144926</v>
+      </c>
+      <c r="DY27">
+        <v>0</v>
+      </c>
+      <c r="DZ27">
+        <v>0</v>
+      </c>
+      <c r="EA27">
+        <v>11920144926</v>
+      </c>
+      <c r="EB27">
+        <v>11920144926</v>
+      </c>
+      <c r="EC27">
+        <v>1102922205</v>
+      </c>
+      <c r="ED27">
+        <v>1102922205</v>
+      </c>
+      <c r="EE27">
+        <v>162299941.19999999</v>
+      </c>
+      <c r="EF27">
+        <v>162299941.19999999</v>
+      </c>
+      <c r="EG27">
+        <v>1929622297</v>
+      </c>
+      <c r="EH27">
+        <v>1929622297</v>
       </c>
       <c r="EJ27">
-        <v>2</v>
+        <v>9999422223</v>
       </c>
       <c r="EK27">
-        <v>2</v>
+        <v>9999422223</v>
       </c>
       <c r="EM27" s="1"/>
     </row>
     <row r="28" spans="1:143" x14ac:dyDescent="0.25">
-      <c r="C28">
-        <v>81007188</v>
-      </c>
       <c r="D28">
-        <v>5000</v>
-      </c>
-      <c r="E28" t="s">
-        <v>159</v>
+        <v>7003</v>
+      </c>
+      <c r="F28" t="s">
+        <v>242</v>
       </c>
       <c r="H28" s="1"/>
       <c r="I28" s="1"/>
-      <c r="L28">
-        <v>971779</v>
-      </c>
-      <c r="M28">
-        <v>971779</v>
-      </c>
-      <c r="N28">
-        <v>2</v>
-      </c>
-      <c r="O28" t="s">
-        <v>202</v>
-      </c>
       <c r="S28">
-        <v>44112081</v>
-      </c>
-      <c r="T28" t="s">
-        <v>210</v>
+        <v>14008840</v>
       </c>
       <c r="AM28" s="1"/>
       <c r="BF28" s="1"/>
-      <c r="BX28">
-        <v>786282668</v>
-      </c>
-      <c r="BY28">
-        <v>97927882</v>
-      </c>
-      <c r="BZ28">
-        <v>96</v>
-      </c>
-      <c r="CA28" t="s">
-        <v>182</v>
-      </c>
       <c r="CB28" s="1"/>
       <c r="CC28" s="1"/>
-      <c r="CD28" t="s">
-        <v>183</v>
-      </c>
-      <c r="CE28">
-        <v>62268</v>
-      </c>
-      <c r="CF28">
-        <v>62268</v>
-      </c>
-      <c r="CG28">
-        <v>2.276672</v>
-      </c>
-      <c r="CH28">
-        <v>769.88</v>
-      </c>
-      <c r="CI28">
-        <v>2.9</v>
-      </c>
-      <c r="CJ28">
-        <v>2</v>
-      </c>
-      <c r="CK28">
-        <v>2</v>
-      </c>
-      <c r="CL28" t="s">
-        <v>171</v>
-      </c>
-      <c r="CM28" t="s">
-        <v>171</v>
-      </c>
-      <c r="CN28">
-        <v>2</v>
-      </c>
       <c r="CO28" s="1"/>
       <c r="CP28" s="1"/>
-      <c r="CS28" t="s">
-        <v>165</v>
-      </c>
-      <c r="CT28" t="s">
-        <v>209</v>
+      <c r="CW28">
+        <v>196414963</v>
+      </c>
+      <c r="CX28">
+        <v>2626291200</v>
+      </c>
+      <c r="DO28">
+        <v>10409999.210000001</v>
+      </c>
+      <c r="DP28">
+        <v>6911299130</v>
+      </c>
+      <c r="DQ28">
+        <v>40246419.020000003</v>
+      </c>
+      <c r="DR28">
+        <v>1961909125</v>
+      </c>
+      <c r="DS28">
+        <v>4964246.6900000004</v>
+      </c>
+      <c r="DT28">
+        <v>4964246.6900000004</v>
+      </c>
+      <c r="DW28">
+        <v>22262666.960000001</v>
+      </c>
+      <c r="DX28">
+        <v>1622242901</v>
+      </c>
+      <c r="DY28">
+        <v>0</v>
+      </c>
+      <c r="DZ28">
+        <v>0</v>
+      </c>
+      <c r="EA28">
+        <v>22262666.960000001</v>
+      </c>
+      <c r="EB28">
+        <v>1622242901</v>
+      </c>
+      <c r="EC28">
+        <v>6642212.96</v>
+      </c>
+      <c r="ED28">
+        <v>126226091.3</v>
+      </c>
+      <c r="EE28">
+        <v>1912.96</v>
+      </c>
+      <c r="EF28">
+        <v>96162.04</v>
+      </c>
+      <c r="EG28">
+        <v>6644220.4900000002</v>
+      </c>
+      <c r="EH28">
+        <v>126119929.7</v>
       </c>
       <c r="EJ28">
-        <v>2</v>
+        <v>26912166.02</v>
       </c>
       <c r="EK28">
-        <v>2</v>
+        <v>1190422929</v>
       </c>
       <c r="EM28" s="1"/>
     </row>
     <row r="29" spans="1:143" x14ac:dyDescent="0.25">
-      <c r="C29">
-        <v>81007188</v>
-      </c>
       <c r="D29">
-        <v>5000</v>
-      </c>
-      <c r="E29" t="s">
-        <v>159</v>
+        <v>7003</v>
+      </c>
+      <c r="F29" t="s">
+        <v>229</v>
       </c>
       <c r="H29" s="1"/>
       <c r="I29" s="1"/>
-      <c r="L29">
-        <v>971779</v>
-      </c>
-      <c r="M29">
-        <v>971779</v>
-      </c>
-      <c r="N29">
-        <v>2</v>
-      </c>
-      <c r="O29" t="s">
-        <v>202</v>
-      </c>
       <c r="S29">
-        <v>44112081</v>
-      </c>
-      <c r="T29" t="s">
-        <v>210</v>
+        <v>14008840</v>
       </c>
       <c r="AM29" s="1"/>
       <c r="BF29" s="1"/>
-      <c r="BX29">
-        <v>728967786</v>
-      </c>
-      <c r="BY29">
-        <v>86877288</v>
-      </c>
-      <c r="BZ29">
-        <v>96</v>
-      </c>
-      <c r="CA29" t="s">
-        <v>182</v>
-      </c>
       <c r="CB29" s="1"/>
       <c r="CC29" s="1"/>
-      <c r="CD29" t="s">
-        <v>183</v>
-      </c>
-      <c r="CE29">
-        <v>79872</v>
-      </c>
-      <c r="CF29">
-        <v>79872</v>
-      </c>
-      <c r="CG29">
-        <v>2.276672</v>
-      </c>
-      <c r="CH29">
-        <v>9768.9599999999991</v>
-      </c>
-      <c r="CI29">
-        <v>2.9</v>
-      </c>
-      <c r="CJ29">
-        <v>2</v>
-      </c>
-      <c r="CK29">
-        <v>2</v>
-      </c>
-      <c r="CL29" t="s">
-        <v>171</v>
-      </c>
-      <c r="CM29" t="s">
-        <v>171</v>
-      </c>
-      <c r="CN29">
-        <v>2</v>
-      </c>
       <c r="CO29" s="1"/>
       <c r="CP29" s="1"/>
-      <c r="CS29" t="s">
-        <v>165</v>
-      </c>
-      <c r="CT29" t="s">
-        <v>209</v>
+      <c r="CW29">
+        <v>641296994.29999995</v>
+      </c>
+      <c r="CX29">
+        <v>14699610997</v>
+      </c>
+      <c r="DO29">
+        <v>119160966.09999999</v>
+      </c>
+      <c r="DP29">
+        <v>2122900611</v>
+      </c>
+      <c r="DQ29">
+        <v>161196296</v>
+      </c>
+      <c r="DR29">
+        <v>6216142044</v>
+      </c>
+      <c r="DS29">
+        <v>9441440</v>
+      </c>
+      <c r="DT29">
+        <v>6201169.2000000002</v>
+      </c>
+      <c r="DW29">
+        <v>99492692.189999998</v>
+      </c>
+      <c r="DX29">
+        <v>4116649923</v>
+      </c>
+      <c r="DY29">
+        <v>0</v>
+      </c>
+      <c r="DZ29">
+        <v>0</v>
+      </c>
+      <c r="EA29">
+        <v>99492692.189999998</v>
+      </c>
+      <c r="EB29">
+        <v>4116649923</v>
+      </c>
+      <c r="EC29">
+        <v>64696442.289999999</v>
+      </c>
+      <c r="ED29">
+        <v>1446622123</v>
+      </c>
+      <c r="EE29">
+        <v>9292194.9000000004</v>
+      </c>
+      <c r="EF29">
+        <v>244099942.5</v>
+      </c>
+      <c r="EG29">
+        <v>40194292.189999998</v>
+      </c>
+      <c r="EH29">
+        <v>1612611665</v>
       </c>
       <c r="EJ29">
-        <v>2</v>
+        <v>99266699</v>
       </c>
       <c r="EK29">
-        <v>2</v>
+        <v>2491961612</v>
       </c>
       <c r="EM29" s="1"/>
     </row>
     <row r="30" spans="1:143" x14ac:dyDescent="0.25">
-      <c r="A30">
-        <v>13</v>
-      </c>
-      <c r="B30" t="s">
-        <v>215</v>
-      </c>
-      <c r="C30">
-        <v>4814314</v>
-      </c>
       <c r="D30">
-        <v>7150</v>
-      </c>
-      <c r="E30" t="s">
-        <v>159</v>
-      </c>
-      <c r="H30" s="1">
-        <v>40648</v>
-      </c>
-      <c r="I30" s="1">
-        <v>40908</v>
-      </c>
-      <c r="J30" t="s">
-        <v>160</v>
-      </c>
-      <c r="K30">
-        <v>1000091</v>
-      </c>
-      <c r="L30">
-        <v>814894</v>
-      </c>
-      <c r="M30">
-        <v>814894</v>
-      </c>
-      <c r="N30">
-        <v>2</v>
-      </c>
-      <c r="O30" t="s">
-        <v>216</v>
-      </c>
-      <c r="P30" t="s">
-        <v>217</v>
-      </c>
-      <c r="Q30">
-        <v>804</v>
-      </c>
-      <c r="R30" t="s">
-        <v>218</v>
-      </c>
+        <v>7003</v>
+      </c>
+      <c r="F30" t="s">
+        <v>243</v>
+      </c>
+      <c r="H30" s="1"/>
+      <c r="I30" s="1"/>
       <c r="S30">
-        <v>15918889</v>
-      </c>
-      <c r="T30" t="s">
-        <v>219</v>
-      </c>
-      <c r="U30" t="s">
-        <v>165</v>
-      </c>
-      <c r="W30" t="s">
-        <v>166</v>
-      </c>
-      <c r="Y30">
-        <v>0</v>
-      </c>
-      <c r="Z30">
-        <v>0</v>
-      </c>
-      <c r="AA30" t="s">
-        <v>167</v>
-      </c>
-      <c r="AB30">
-        <v>142</v>
-      </c>
-      <c r="AF30" t="s">
-        <v>220</v>
-      </c>
-      <c r="AG30">
-        <v>0</v>
-      </c>
-      <c r="AH30">
-        <v>0</v>
-      </c>
-      <c r="AK30">
-        <v>9</v>
-      </c>
-      <c r="AL30">
-        <v>9</v>
+        <v>14008840</v>
       </c>
       <c r="AM30" s="1"/>
-      <c r="AN30">
-        <v>8</v>
-      </c>
-      <c r="AO30">
-        <v>8</v>
-      </c>
-      <c r="AP30" t="s">
-        <v>171</v>
-      </c>
-      <c r="AQ30" t="s">
-        <v>171</v>
-      </c>
-      <c r="AW30" t="s">
-        <v>171</v>
-      </c>
-      <c r="BB30" t="s">
-        <v>171</v>
-      </c>
-      <c r="BC30" t="s">
-        <v>165</v>
-      </c>
-      <c r="BD30" t="s">
-        <v>165</v>
-      </c>
-      <c r="BE30">
-        <v>6</v>
-      </c>
       <c r="BF30" s="1"/>
-      <c r="BG30" t="s">
-        <v>221</v>
-      </c>
-      <c r="BH30" t="s">
-        <v>172</v>
-      </c>
-      <c r="BI30">
-        <v>69</v>
-      </c>
-      <c r="BM30" t="s">
-        <v>171</v>
-      </c>
-      <c r="BN30" t="s">
-        <v>222</v>
-      </c>
-      <c r="BO30">
-        <v>62</v>
-      </c>
-      <c r="BS30">
-        <v>62</v>
-      </c>
-      <c r="BT30">
-        <v>6</v>
-      </c>
       <c r="CB30" s="1"/>
       <c r="CC30" s="1"/>
-      <c r="CL30" t="s">
-        <v>171</v>
-      </c>
-      <c r="CM30" t="s">
-        <v>171</v>
-      </c>
-      <c r="CN30">
-        <v>2</v>
-      </c>
       <c r="CO30" s="1"/>
       <c r="CP30" s="1"/>
-      <c r="CV30">
-        <v>2</v>
-      </c>
-      <c r="CW30">
-        <v>669222</v>
-      </c>
       <c r="CX30">
-        <v>669222</v>
-      </c>
-      <c r="CY30">
-        <v>669222</v>
-      </c>
-      <c r="CZ30">
-        <v>669222</v>
-      </c>
-      <c r="DW30">
-        <v>669222</v>
+        <v>22621264602</v>
+      </c>
+      <c r="DP30">
+        <v>96029412030</v>
+      </c>
+      <c r="DR30">
+        <v>44426012423</v>
+      </c>
+      <c r="DT30">
+        <v>201962999</v>
+      </c>
+      <c r="DV30">
+        <v>2161.91</v>
       </c>
       <c r="DX30">
-        <v>669222</v>
-      </c>
-      <c r="DY30">
-        <v>2</v>
+        <v>12014242405</v>
       </c>
       <c r="DZ30">
-        <v>2</v>
-      </c>
-      <c r="EA30">
-        <v>669222</v>
+        <v>0</v>
       </c>
       <c r="EB30">
-        <v>669222</v>
-      </c>
-      <c r="EG30">
-        <v>2</v>
+        <v>12014242405</v>
+      </c>
+      <c r="ED30">
+        <v>6422912119</v>
+      </c>
+      <c r="EF30">
+        <v>411999991.69999999</v>
       </c>
       <c r="EH30">
-        <v>2</v>
-      </c>
-      <c r="EJ30">
-        <v>669222</v>
+        <v>6169126146</v>
       </c>
       <c r="EK30">
-        <v>669222</v>
-      </c>
-      <c r="EL30" t="s">
-        <v>174</v>
+        <v>16244161960</v>
       </c>
       <c r="EM30" s="1"/>
-    </row>
-    <row r="31" spans="1:143" x14ac:dyDescent="0.25">
-      <c r="A31">
-        <v>14</v>
-      </c>
-      <c r="B31" t="s">
-        <v>223</v>
-      </c>
-      <c r="C31">
-        <v>4811010</v>
-      </c>
-      <c r="D31">
-        <v>7150</v>
-      </c>
-      <c r="E31" t="s">
-        <v>159</v>
-      </c>
-      <c r="H31" s="1">
-        <v>37068</v>
-      </c>
-      <c r="I31" s="1">
-        <v>40908</v>
-      </c>
-      <c r="J31" t="s">
-        <v>160</v>
-      </c>
-      <c r="K31">
-        <v>1000091</v>
-      </c>
-      <c r="L31">
-        <v>814894</v>
-      </c>
-      <c r="M31">
-        <v>814894</v>
-      </c>
-      <c r="N31">
-        <v>2</v>
-      </c>
-      <c r="O31" t="s">
-        <v>216</v>
-      </c>
-      <c r="P31" t="s">
-        <v>217</v>
-      </c>
-      <c r="Q31">
-        <v>804</v>
-      </c>
-      <c r="R31" t="s">
-        <v>218</v>
-      </c>
-      <c r="S31">
-        <v>15918889</v>
-      </c>
-      <c r="T31" t="s">
-        <v>219</v>
-      </c>
-      <c r="U31" t="s">
-        <v>165</v>
-      </c>
-      <c r="W31" t="s">
-        <v>166</v>
-      </c>
-      <c r="Y31">
-        <v>0</v>
-      </c>
-      <c r="Z31">
-        <v>0</v>
-      </c>
-      <c r="AA31" t="s">
-        <v>167</v>
-      </c>
-      <c r="AB31">
-        <v>142</v>
-      </c>
-      <c r="AF31" t="s">
-        <v>224</v>
-      </c>
-      <c r="AG31">
-        <v>0</v>
-      </c>
-      <c r="AH31">
-        <v>0</v>
-      </c>
-      <c r="AK31">
-        <v>9</v>
-      </c>
-      <c r="AL31">
-        <v>9</v>
-      </c>
-      <c r="AM31" s="1"/>
-      <c r="AN31">
-        <v>8</v>
-      </c>
-      <c r="AO31">
-        <v>8</v>
-      </c>
-      <c r="AP31" t="s">
-        <v>171</v>
-      </c>
-      <c r="AQ31" t="s">
-        <v>171</v>
-      </c>
-      <c r="AW31" t="s">
-        <v>171</v>
-      </c>
-      <c r="BB31" t="s">
-        <v>171</v>
-      </c>
-      <c r="BC31" t="s">
-        <v>165</v>
-      </c>
-      <c r="BD31" t="s">
-        <v>165</v>
-      </c>
-      <c r="BE31">
-        <v>6</v>
-      </c>
-      <c r="BF31" s="1"/>
-      <c r="BG31" t="s">
-        <v>221</v>
-      </c>
-      <c r="BH31" t="s">
-        <v>172</v>
-      </c>
-      <c r="BI31">
-        <v>69</v>
-      </c>
-      <c r="BM31" t="s">
-        <v>171</v>
-      </c>
-      <c r="BN31" t="s">
-        <v>222</v>
-      </c>
-      <c r="BO31">
-        <v>62</v>
-      </c>
-      <c r="BS31">
-        <v>62</v>
-      </c>
-      <c r="BT31">
-        <v>6</v>
-      </c>
-      <c r="CB31" s="1"/>
-      <c r="CC31" s="1"/>
-      <c r="CL31" t="s">
-        <v>171</v>
-      </c>
-      <c r="CM31" t="s">
-        <v>171</v>
-      </c>
-      <c r="CN31">
-        <v>2</v>
-      </c>
-      <c r="CO31" s="1"/>
-      <c r="CP31" s="1"/>
-      <c r="CV31">
-        <v>2</v>
-      </c>
-      <c r="CW31">
-        <v>7672222</v>
-      </c>
-      <c r="CX31">
-        <v>7672222</v>
-      </c>
-      <c r="CY31">
-        <v>7672222</v>
-      </c>
-      <c r="CZ31">
-        <v>7672222</v>
-      </c>
-      <c r="DW31">
-        <v>7672222</v>
-      </c>
-      <c r="DX31">
-        <v>7672222</v>
-      </c>
-      <c r="DY31">
-        <v>2</v>
-      </c>
-      <c r="DZ31">
-        <v>2</v>
-      </c>
-      <c r="EA31">
-        <v>7672222</v>
-      </c>
-      <c r="EB31">
-        <v>7672222</v>
-      </c>
-      <c r="EG31">
-        <v>2</v>
-      </c>
-      <c r="EH31">
-        <v>2</v>
-      </c>
-      <c r="EJ31">
-        <v>7672222</v>
-      </c>
-      <c r="EK31">
-        <v>7672222</v>
-      </c>
-      <c r="EL31" t="s">
-        <v>174</v>
-      </c>
-      <c r="EM31" s="1"/>
-    </row>
-    <row r="32" spans="1:143" x14ac:dyDescent="0.25">
-      <c r="A32">
-        <v>15</v>
-      </c>
-      <c r="B32" t="s">
-        <v>225</v>
-      </c>
-      <c r="C32">
-        <v>104111348</v>
-      </c>
-      <c r="D32">
-        <v>7160</v>
-      </c>
-      <c r="E32" t="s">
-        <v>176</v>
-      </c>
-      <c r="H32" s="1">
-        <v>45965</v>
-      </c>
-      <c r="I32" s="1">
-        <v>46057</v>
-      </c>
-      <c r="J32" t="s">
-        <v>160</v>
-      </c>
-      <c r="K32">
-        <v>1000091</v>
-      </c>
-      <c r="L32">
-        <v>811681</v>
-      </c>
-      <c r="M32">
-        <v>811681</v>
-      </c>
-      <c r="N32">
-        <v>1</v>
-      </c>
-      <c r="O32" t="s">
-        <v>226</v>
-      </c>
-      <c r="Q32">
-        <v>804</v>
-      </c>
-      <c r="R32" t="s">
-        <v>163</v>
-      </c>
-      <c r="S32">
-        <v>154108</v>
-      </c>
-      <c r="T32" t="s">
-        <v>227</v>
-      </c>
-      <c r="U32" t="s">
-        <v>165</v>
-      </c>
-      <c r="W32" t="s">
-        <v>166</v>
-      </c>
-      <c r="Y32">
-        <v>0</v>
-      </c>
-      <c r="AA32" t="s">
-        <v>167</v>
-      </c>
-      <c r="AB32">
-        <v>182</v>
-      </c>
-      <c r="AF32" t="s">
-        <v>228</v>
-      </c>
-      <c r="AG32">
-        <v>0</v>
-      </c>
-      <c r="AH32">
-        <v>0</v>
-      </c>
-      <c r="AK32">
-        <v>9</v>
-      </c>
-      <c r="AL32">
-        <v>9</v>
-      </c>
-      <c r="AM32" s="1"/>
-      <c r="AO32">
-        <v>9</v>
-      </c>
-      <c r="AP32" t="s">
-        <v>171</v>
-      </c>
-      <c r="AQ32" t="s">
-        <v>171</v>
-      </c>
-      <c r="AW32" t="s">
-        <v>171</v>
-      </c>
-      <c r="BB32" t="s">
-        <v>171</v>
-      </c>
-      <c r="BC32" t="s">
-        <v>171</v>
-      </c>
-      <c r="BD32" t="s">
-        <v>171</v>
-      </c>
-      <c r="BF32" s="1"/>
-      <c r="BH32" t="s">
-        <v>172</v>
-      </c>
-      <c r="BJ32">
-        <v>9</v>
-      </c>
-      <c r="BM32" t="s">
-        <v>171</v>
-      </c>
-      <c r="BP32">
-        <v>9</v>
-      </c>
-      <c r="BS32">
-        <v>9</v>
-      </c>
-      <c r="BV32">
-        <v>6</v>
-      </c>
-      <c r="BY32">
-        <v>69989976</v>
-      </c>
-      <c r="BZ32">
-        <v>76</v>
-      </c>
-      <c r="CA32" t="s">
-        <v>182</v>
-      </c>
-      <c r="CB32" s="1"/>
-      <c r="CC32" s="1"/>
-      <c r="CD32" t="s">
-        <v>183</v>
-      </c>
-      <c r="CE32">
-        <v>2</v>
-      </c>
-      <c r="CF32">
-        <v>2</v>
-      </c>
-      <c r="CG32">
-        <v>6</v>
-      </c>
-      <c r="CH32">
-        <v>2</v>
-      </c>
-      <c r="CI32">
-        <v>6</v>
-      </c>
-      <c r="CJ32">
-        <v>2</v>
-      </c>
-      <c r="CK32">
-        <v>2</v>
-      </c>
-      <c r="CL32" t="s">
-        <v>171</v>
-      </c>
-      <c r="CM32" t="s">
-        <v>171</v>
-      </c>
-      <c r="CN32">
-        <v>92.29</v>
-      </c>
-      <c r="CO32" s="1"/>
-      <c r="CP32" s="1"/>
-      <c r="CS32" t="s">
-        <v>171</v>
-      </c>
-      <c r="CV32">
-        <v>2</v>
-      </c>
-      <c r="DO32">
-        <v>87766829.989999995</v>
-      </c>
-      <c r="DP32">
-        <v>87766829.989999995</v>
-      </c>
-      <c r="DQ32">
-        <v>87727287.680000007</v>
-      </c>
-      <c r="DR32">
-        <v>87727287.680000007</v>
-      </c>
-      <c r="DS32">
-        <v>87766.86</v>
-      </c>
-      <c r="DT32">
-        <v>87766.86</v>
-      </c>
-      <c r="DY32">
-        <v>2</v>
-      </c>
-      <c r="DZ32">
-        <v>2</v>
-      </c>
-      <c r="EA32">
-        <v>2</v>
-      </c>
-      <c r="EB32">
-        <v>2</v>
-      </c>
-      <c r="EG32">
-        <v>2</v>
-      </c>
-      <c r="EH32">
-        <v>2</v>
-      </c>
-      <c r="EJ32">
-        <v>2</v>
-      </c>
-      <c r="EK32">
-        <v>2</v>
-      </c>
-      <c r="EL32" t="s">
-        <v>174</v>
-      </c>
-      <c r="EM32" s="1"/>
-    </row>
-    <row r="33" spans="1:143" x14ac:dyDescent="0.25">
-      <c r="A33">
-        <v>16</v>
-      </c>
-      <c r="B33" t="s">
-        <v>229</v>
-      </c>
-      <c r="C33">
-        <v>104414770</v>
-      </c>
-      <c r="D33">
-        <v>7160</v>
-      </c>
-      <c r="E33" t="s">
-        <v>176</v>
-      </c>
-      <c r="H33" s="1">
-        <v>45965</v>
-      </c>
-      <c r="I33" s="1">
-        <v>46052</v>
-      </c>
-      <c r="J33" t="s">
-        <v>160</v>
-      </c>
-      <c r="K33">
-        <v>1000091</v>
-      </c>
-      <c r="L33">
-        <v>811681</v>
-      </c>
-      <c r="M33">
-        <v>811681</v>
-      </c>
-      <c r="N33">
-        <v>1</v>
-      </c>
-      <c r="O33" t="s">
-        <v>226</v>
-      </c>
-      <c r="Q33">
-        <v>804</v>
-      </c>
-      <c r="R33" t="s">
-        <v>163</v>
-      </c>
-      <c r="S33">
-        <v>154108</v>
-      </c>
-      <c r="T33" t="s">
-        <v>227</v>
-      </c>
-      <c r="U33" t="s">
-        <v>165</v>
-      </c>
-      <c r="W33" t="s">
-        <v>166</v>
-      </c>
-      <c r="Y33">
-        <v>0</v>
-      </c>
-      <c r="AA33" t="s">
-        <v>167</v>
-      </c>
-      <c r="AB33">
-        <v>182</v>
-      </c>
-      <c r="AF33" t="s">
-        <v>230</v>
-      </c>
-      <c r="AG33">
-        <v>0</v>
-      </c>
-      <c r="AH33">
-        <v>0</v>
-      </c>
-      <c r="AK33">
-        <v>9</v>
-      </c>
-      <c r="AL33">
-        <v>9</v>
-      </c>
-      <c r="AM33" s="1"/>
-      <c r="AO33">
-        <v>9</v>
-      </c>
-      <c r="AP33" t="s">
-        <v>171</v>
-      </c>
-      <c r="AQ33" t="s">
-        <v>171</v>
-      </c>
-      <c r="AW33" t="s">
-        <v>171</v>
-      </c>
-      <c r="BB33" t="s">
-        <v>171</v>
-      </c>
-      <c r="BC33" t="s">
-        <v>171</v>
-      </c>
-      <c r="BD33" t="s">
-        <v>171</v>
-      </c>
-      <c r="BF33" s="1"/>
-      <c r="BH33" t="s">
-        <v>172</v>
-      </c>
-      <c r="BJ33">
-        <v>9</v>
-      </c>
-      <c r="BM33" t="s">
-        <v>171</v>
-      </c>
-      <c r="BP33">
-        <v>9</v>
-      </c>
-      <c r="BS33">
-        <v>9</v>
-      </c>
-      <c r="BV33">
-        <v>6</v>
-      </c>
-      <c r="BY33">
-        <v>69989976</v>
-      </c>
-      <c r="BZ33">
-        <v>76</v>
-      </c>
-      <c r="CA33" t="s">
-        <v>182</v>
-      </c>
-      <c r="CB33" s="1"/>
-      <c r="CC33" s="1"/>
-      <c r="CD33" t="s">
-        <v>183</v>
-      </c>
-      <c r="CE33">
-        <v>2</v>
-      </c>
-      <c r="CF33">
-        <v>2</v>
-      </c>
-      <c r="CG33">
-        <v>6</v>
-      </c>
-      <c r="CH33">
-        <v>2</v>
-      </c>
-      <c r="CI33">
-        <v>6</v>
-      </c>
-      <c r="CJ33">
-        <v>2</v>
-      </c>
-      <c r="CK33">
-        <v>2</v>
-      </c>
-      <c r="CL33" t="s">
-        <v>171</v>
-      </c>
-      <c r="CM33" t="s">
-        <v>171</v>
-      </c>
-      <c r="CN33">
-        <v>92.29</v>
-      </c>
-      <c r="CO33" s="1"/>
-      <c r="CP33" s="1"/>
-      <c r="CS33" t="s">
-        <v>171</v>
-      </c>
-      <c r="CV33">
-        <v>2</v>
-      </c>
-      <c r="DO33">
-        <v>8677286.9600000009</v>
-      </c>
-      <c r="DP33">
-        <v>8677286.9600000009</v>
-      </c>
-      <c r="DQ33">
-        <v>8668628.6699999999</v>
-      </c>
-      <c r="DR33">
-        <v>8668628.6699999999</v>
-      </c>
-      <c r="DS33">
-        <v>8677.2800000000007</v>
-      </c>
-      <c r="DT33">
-        <v>8677.2800000000007</v>
-      </c>
-      <c r="DY33">
-        <v>2</v>
-      </c>
-      <c r="DZ33">
-        <v>2</v>
-      </c>
-      <c r="EA33">
-        <v>2</v>
-      </c>
-      <c r="EB33">
-        <v>2</v>
-      </c>
-      <c r="EG33">
-        <v>2</v>
-      </c>
-      <c r="EH33">
-        <v>2</v>
-      </c>
-      <c r="EJ33">
-        <v>2</v>
-      </c>
-      <c r="EK33">
-        <v>2</v>
-      </c>
-      <c r="EL33" t="s">
-        <v>174</v>
-      </c>
-      <c r="EM33" s="1"/>
-    </row>
-    <row r="34" spans="1:143" x14ac:dyDescent="0.25">
-      <c r="A34">
-        <v>17</v>
-      </c>
-      <c r="B34" t="s">
-        <v>231</v>
-      </c>
-      <c r="C34">
-        <v>88441027</v>
-      </c>
-      <c r="D34">
-        <v>7003</v>
-      </c>
-      <c r="E34" t="s">
-        <v>176</v>
-      </c>
-      <c r="F34" t="s">
-        <v>232</v>
-      </c>
-      <c r="G34">
-        <v>42.094799999999999</v>
-      </c>
-      <c r="H34" s="1">
-        <v>45763</v>
-      </c>
-      <c r="I34" s="1">
-        <v>46024</v>
-      </c>
-      <c r="J34" t="s">
-        <v>160</v>
-      </c>
-      <c r="K34">
-        <v>1000091</v>
-      </c>
-      <c r="L34">
-        <v>867006</v>
-      </c>
-      <c r="M34">
-        <v>867006</v>
-      </c>
-      <c r="N34">
-        <v>2</v>
-      </c>
-      <c r="O34" t="s">
-        <v>233</v>
-      </c>
-      <c r="P34" t="s">
-        <v>203</v>
-      </c>
-      <c r="Q34">
-        <v>804</v>
-      </c>
-      <c r="R34" t="s">
-        <v>163</v>
-      </c>
-      <c r="S34">
-        <v>14008840</v>
-      </c>
-      <c r="T34" t="s">
-        <v>234</v>
-      </c>
-      <c r="U34" t="s">
-        <v>165</v>
-      </c>
-      <c r="W34" t="s">
-        <v>166</v>
-      </c>
-      <c r="Y34">
-        <v>0</v>
-      </c>
-      <c r="Z34">
-        <v>85.8</v>
-      </c>
-      <c r="AA34" t="s">
-        <v>167</v>
-      </c>
-      <c r="AB34">
-        <v>221</v>
-      </c>
-      <c r="AF34" t="s">
-        <v>235</v>
-      </c>
-      <c r="AG34">
-        <v>0</v>
-      </c>
-      <c r="AH34">
-        <v>0</v>
-      </c>
-      <c r="AI34">
-        <v>0</v>
-      </c>
-      <c r="AK34">
-        <v>8.9</v>
-      </c>
-      <c r="AL34">
-        <v>8.9</v>
-      </c>
-      <c r="AM34" s="1"/>
-      <c r="AN34">
-        <v>6</v>
-      </c>
-      <c r="AO34">
-        <v>2</v>
-      </c>
-      <c r="AP34" t="s">
-        <v>171</v>
-      </c>
-      <c r="AQ34" t="s">
-        <v>165</v>
-      </c>
-      <c r="AR34">
-        <v>267226</v>
-      </c>
-      <c r="AS34" t="s">
-        <v>236</v>
-      </c>
-      <c r="AT34">
-        <v>2</v>
-      </c>
-      <c r="AU34">
-        <v>2</v>
-      </c>
-      <c r="AW34" t="s">
-        <v>171</v>
-      </c>
-      <c r="BB34" t="s">
-        <v>171</v>
-      </c>
-      <c r="BC34" t="s">
-        <v>171</v>
-      </c>
-      <c r="BD34" t="s">
-        <v>171</v>
-      </c>
-      <c r="BF34" s="1"/>
-      <c r="BG34" t="s">
-        <v>237</v>
-      </c>
-      <c r="BH34" t="s">
-        <v>172</v>
-      </c>
-      <c r="BJ34">
-        <v>2</v>
-      </c>
-      <c r="BM34" t="s">
-        <v>171</v>
-      </c>
-      <c r="BN34" t="s">
-        <v>238</v>
-      </c>
-      <c r="BP34">
-        <v>2</v>
-      </c>
-      <c r="BS34">
-        <v>2</v>
-      </c>
-      <c r="BT34">
-        <v>2.2698</v>
-      </c>
-      <c r="BV34">
-        <v>6</v>
-      </c>
-      <c r="BX34">
-        <v>787688828</v>
-      </c>
-      <c r="BY34">
-        <v>98986787</v>
-      </c>
-      <c r="BZ34">
-        <v>96</v>
-      </c>
-      <c r="CA34" t="s">
-        <v>182</v>
-      </c>
-      <c r="CB34" s="1"/>
-      <c r="CC34" s="1"/>
-      <c r="CD34" t="s">
-        <v>183</v>
-      </c>
-      <c r="CE34">
-        <v>682228</v>
-      </c>
-      <c r="CF34">
-        <v>682228</v>
-      </c>
-      <c r="CG34">
-        <v>2.2887680000000001</v>
-      </c>
-      <c r="CH34">
-        <v>96879.89</v>
-      </c>
-      <c r="CI34">
-        <v>2.9</v>
-      </c>
-      <c r="CJ34">
-        <v>2</v>
-      </c>
-      <c r="CK34">
-        <v>2</v>
-      </c>
-      <c r="CL34" t="s">
-        <v>171</v>
-      </c>
-      <c r="CM34" t="s">
-        <v>171</v>
-      </c>
-      <c r="CN34">
-        <v>2</v>
-      </c>
-      <c r="CO34" s="1"/>
-      <c r="CP34" s="1"/>
-      <c r="CS34" t="s">
-        <v>165</v>
-      </c>
-      <c r="CT34" t="s">
-        <v>211</v>
-      </c>
-      <c r="CV34">
-        <v>2</v>
-      </c>
-      <c r="DO34">
-        <v>927696.66</v>
-      </c>
-      <c r="DP34">
-        <v>22226962.789999999</v>
-      </c>
-      <c r="DQ34">
-        <v>927696.66</v>
-      </c>
-      <c r="DR34">
-        <v>22226962.789999999</v>
-      </c>
-      <c r="DW34">
-        <v>62689.68</v>
-      </c>
-      <c r="DX34">
-        <v>827226.22</v>
-      </c>
-      <c r="DY34">
-        <v>2</v>
-      </c>
-      <c r="DZ34">
-        <v>2</v>
-      </c>
-      <c r="EA34">
-        <v>62689.68</v>
-      </c>
-      <c r="EB34">
-        <v>827226.22</v>
-      </c>
-      <c r="EG34">
-        <v>2</v>
-      </c>
-      <c r="EH34">
-        <v>2</v>
-      </c>
-      <c r="EJ34">
-        <v>62689.68</v>
-      </c>
-      <c r="EK34">
-        <v>827226.22</v>
-      </c>
-      <c r="EL34" t="s">
-        <v>174</v>
-      </c>
-      <c r="EM34" s="1"/>
-    </row>
-    <row r="35" spans="1:143" x14ac:dyDescent="0.25">
-      <c r="A35">
-        <v>18</v>
-      </c>
-      <c r="B35" t="s">
-        <v>239</v>
-      </c>
-      <c r="C35">
-        <v>100243246</v>
-      </c>
-      <c r="D35">
-        <v>7003</v>
-      </c>
-      <c r="E35" t="s">
-        <v>176</v>
-      </c>
-      <c r="F35" t="s">
-        <v>232</v>
-      </c>
-      <c r="G35">
-        <v>42.094799999999999</v>
-      </c>
-      <c r="H35" s="1">
-        <v>45690</v>
-      </c>
-      <c r="I35" s="1">
-        <v>46024</v>
-      </c>
-      <c r="J35" t="s">
-        <v>160</v>
-      </c>
-      <c r="K35">
-        <v>1000091</v>
-      </c>
-      <c r="L35">
-        <v>867006</v>
-      </c>
-      <c r="M35">
-        <v>867006</v>
-      </c>
-      <c r="N35">
-        <v>2</v>
-      </c>
-      <c r="O35" t="s">
-        <v>233</v>
-      </c>
-      <c r="P35" t="s">
-        <v>203</v>
-      </c>
-      <c r="Q35">
-        <v>804</v>
-      </c>
-      <c r="R35" t="s">
-        <v>163</v>
-      </c>
-      <c r="S35">
-        <v>14008840</v>
-      </c>
-      <c r="T35" t="s">
-        <v>234</v>
-      </c>
-      <c r="U35" t="s">
-        <v>165</v>
-      </c>
-      <c r="W35" t="s">
-        <v>166</v>
-      </c>
-      <c r="Y35">
-        <v>0</v>
-      </c>
-      <c r="Z35">
-        <v>85.8</v>
-      </c>
-      <c r="AA35" t="s">
-        <v>167</v>
-      </c>
-      <c r="AB35">
-        <v>221</v>
-      </c>
-      <c r="AF35" t="s">
-        <v>240</v>
-      </c>
-      <c r="AG35">
-        <v>0</v>
-      </c>
-      <c r="AH35">
-        <v>0</v>
-      </c>
-      <c r="AI35">
-        <v>0</v>
-      </c>
-      <c r="AK35">
-        <v>8.9</v>
-      </c>
-      <c r="AL35">
-        <v>8.9</v>
-      </c>
-      <c r="AM35" s="1"/>
-      <c r="AN35">
-        <v>6</v>
-      </c>
-      <c r="AO35">
-        <v>2</v>
-      </c>
-      <c r="AP35" t="s">
-        <v>171</v>
-      </c>
-      <c r="AQ35" t="s">
-        <v>165</v>
-      </c>
-      <c r="AR35">
-        <v>267226</v>
-      </c>
-      <c r="AS35" t="s">
-        <v>236</v>
-      </c>
-      <c r="AT35">
-        <v>2</v>
-      </c>
-      <c r="AU35">
-        <v>2</v>
-      </c>
-      <c r="AW35" t="s">
-        <v>171</v>
-      </c>
-      <c r="BB35" t="s">
-        <v>171</v>
-      </c>
-      <c r="BC35" t="s">
-        <v>171</v>
-      </c>
-      <c r="BD35" t="s">
-        <v>171</v>
-      </c>
-      <c r="BF35" s="1"/>
-      <c r="BG35" t="s">
-        <v>237</v>
-      </c>
-      <c r="BH35" t="s">
-        <v>172</v>
-      </c>
-      <c r="BJ35">
-        <v>2</v>
-      </c>
-      <c r="BM35" t="s">
-        <v>171</v>
-      </c>
-      <c r="BN35" t="s">
-        <v>238</v>
-      </c>
-      <c r="BP35">
-        <v>2</v>
-      </c>
-      <c r="BS35">
-        <v>2</v>
-      </c>
-      <c r="BT35">
-        <v>2.2698</v>
-      </c>
-      <c r="BV35">
-        <v>6</v>
-      </c>
-      <c r="BX35">
-        <v>286979998</v>
-      </c>
-      <c r="BY35">
-        <v>78266622</v>
-      </c>
-      <c r="BZ35">
-        <v>77</v>
-      </c>
-      <c r="CA35" t="s">
-        <v>182</v>
-      </c>
-      <c r="CB35" s="1"/>
-      <c r="CC35" s="1"/>
-      <c r="CD35" t="s">
-        <v>174</v>
-      </c>
-      <c r="CE35">
-        <v>778268229.29999995</v>
-      </c>
-      <c r="CF35">
-        <v>778268229.29999995</v>
-      </c>
-      <c r="CG35">
-        <v>2.6627890000000001</v>
-      </c>
-      <c r="CH35">
-        <v>228698696.90000001</v>
-      </c>
-      <c r="CI35">
-        <v>2.8</v>
-      </c>
-      <c r="CJ35">
-        <v>2</v>
-      </c>
-      <c r="CK35">
-        <v>2</v>
-      </c>
-      <c r="CL35" t="s">
-        <v>171</v>
-      </c>
-      <c r="CM35" t="s">
-        <v>171</v>
-      </c>
-      <c r="CN35">
-        <v>2</v>
-      </c>
-      <c r="CO35" s="1"/>
-      <c r="CP35" s="1"/>
-      <c r="CQ35" t="s">
-        <v>171</v>
-      </c>
-      <c r="CS35" t="s">
-        <v>165</v>
-      </c>
-      <c r="CT35" t="s">
-        <v>214</v>
-      </c>
-      <c r="CV35">
-        <v>2</v>
-      </c>
-      <c r="DO35">
-        <v>62686</v>
-      </c>
-      <c r="DP35">
-        <v>2676862.77</v>
-      </c>
-      <c r="DQ35">
-        <v>62686</v>
-      </c>
-      <c r="DR35">
-        <v>2676862.77</v>
-      </c>
-      <c r="DW35">
-        <v>6269.28</v>
-      </c>
-      <c r="DX35">
-        <v>96699.28</v>
-      </c>
-      <c r="DY35">
-        <v>2</v>
-      </c>
-      <c r="DZ35">
-        <v>2</v>
-      </c>
-      <c r="EA35">
-        <v>6269.28</v>
-      </c>
-      <c r="EB35">
-        <v>96699.28</v>
-      </c>
-      <c r="EG35">
-        <v>2</v>
-      </c>
-      <c r="EH35">
-        <v>2</v>
-      </c>
-      <c r="EJ35">
-        <v>6269.28</v>
-      </c>
-      <c r="EK35">
-        <v>96699.28</v>
-      </c>
-      <c r="EL35" t="s">
-        <v>174</v>
-      </c>
-      <c r="EM35" s="1"/>
-    </row>
-    <row r="36" spans="1:143" x14ac:dyDescent="0.25">
-      <c r="A36">
-        <v>19</v>
-      </c>
-      <c r="B36" t="s">
-        <v>241</v>
-      </c>
-      <c r="C36">
-        <v>100461040</v>
-      </c>
-      <c r="D36">
-        <v>7003</v>
-      </c>
-      <c r="E36" t="s">
-        <v>176</v>
-      </c>
-      <c r="F36" t="s">
-        <v>232</v>
-      </c>
-      <c r="G36">
-        <v>42.094799999999999</v>
-      </c>
-      <c r="H36" s="1">
-        <v>45700</v>
-      </c>
-      <c r="I36" s="1">
-        <v>46017</v>
-      </c>
-      <c r="J36" t="s">
-        <v>160</v>
-      </c>
-      <c r="K36">
-        <v>1000091</v>
-      </c>
-      <c r="L36">
-        <v>867006</v>
-      </c>
-      <c r="M36">
-        <v>867006</v>
-      </c>
-      <c r="N36">
-        <v>2</v>
-      </c>
-      <c r="O36" t="s">
-        <v>233</v>
-      </c>
-      <c r="P36" t="s">
-        <v>203</v>
-      </c>
-      <c r="Q36">
-        <v>804</v>
-      </c>
-      <c r="R36" t="s">
-        <v>163</v>
-      </c>
-      <c r="S36">
-        <v>14008840</v>
-      </c>
-      <c r="T36" t="s">
-        <v>234</v>
-      </c>
-      <c r="U36" t="s">
-        <v>165</v>
-      </c>
-      <c r="W36" t="s">
-        <v>166</v>
-      </c>
-      <c r="Y36">
-        <v>0</v>
-      </c>
-      <c r="Z36">
-        <v>85.8</v>
-      </c>
-      <c r="AA36" t="s">
-        <v>167</v>
-      </c>
-      <c r="AB36">
-        <v>221</v>
-      </c>
-      <c r="AF36" t="s">
-        <v>242</v>
-      </c>
-      <c r="AG36">
-        <v>0</v>
-      </c>
-      <c r="AH36">
-        <v>0</v>
-      </c>
-      <c r="AI36">
-        <v>0</v>
-      </c>
-      <c r="AK36">
-        <v>8.9</v>
-      </c>
-      <c r="AL36">
-        <v>8.9</v>
-      </c>
-      <c r="AM36" s="1"/>
-      <c r="AN36">
-        <v>6</v>
-      </c>
-      <c r="AO36">
-        <v>2</v>
-      </c>
-      <c r="AP36" t="s">
-        <v>171</v>
-      </c>
-      <c r="AQ36" t="s">
-        <v>165</v>
-      </c>
-      <c r="AR36">
-        <v>267226</v>
-      </c>
-      <c r="AS36" t="s">
-        <v>236</v>
-      </c>
-      <c r="AT36">
-        <v>2</v>
-      </c>
-      <c r="AU36">
-        <v>2</v>
-      </c>
-      <c r="AW36" t="s">
-        <v>171</v>
-      </c>
-      <c r="BB36" t="s">
-        <v>171</v>
-      </c>
-      <c r="BC36" t="s">
-        <v>171</v>
-      </c>
-      <c r="BD36" t="s">
-        <v>171</v>
-      </c>
-      <c r="BF36" s="1"/>
-      <c r="BG36" t="s">
-        <v>237</v>
-      </c>
-      <c r="BH36" t="s">
-        <v>172</v>
-      </c>
-      <c r="BJ36">
-        <v>2</v>
-      </c>
-      <c r="BM36" t="s">
-        <v>171</v>
-      </c>
-      <c r="BN36" t="s">
-        <v>238</v>
-      </c>
-      <c r="BP36">
-        <v>2</v>
-      </c>
-      <c r="BS36">
-        <v>2</v>
-      </c>
-      <c r="BT36">
-        <v>2.2698</v>
-      </c>
-      <c r="BV36">
-        <v>6</v>
-      </c>
-      <c r="BX36">
-        <v>787688798</v>
-      </c>
-      <c r="BY36">
-        <v>98986628</v>
-      </c>
-      <c r="BZ36">
-        <v>96</v>
-      </c>
-      <c r="CA36" t="s">
-        <v>182</v>
-      </c>
-      <c r="CB36" s="1"/>
-      <c r="CC36" s="1"/>
-      <c r="CD36" t="s">
-        <v>183</v>
-      </c>
-      <c r="CE36">
-        <v>289866</v>
-      </c>
-      <c r="CF36">
-        <v>289866</v>
-      </c>
-      <c r="CG36">
-        <v>2.2887680000000001</v>
-      </c>
-      <c r="CH36">
-        <v>76278.679999999993</v>
-      </c>
-      <c r="CI36">
-        <v>2.9</v>
-      </c>
-      <c r="CJ36">
-        <v>2</v>
-      </c>
-      <c r="CK36">
-        <v>2</v>
-      </c>
-      <c r="CL36" t="s">
-        <v>171</v>
-      </c>
-      <c r="CM36" t="s">
-        <v>171</v>
-      </c>
-      <c r="CN36">
-        <v>2</v>
-      </c>
-      <c r="CO36" s="1"/>
-      <c r="CP36" s="1"/>
-      <c r="CS36" t="s">
-        <v>165</v>
-      </c>
-      <c r="CT36" t="s">
-        <v>211</v>
-      </c>
-      <c r="CV36">
-        <v>2</v>
-      </c>
-      <c r="DO36">
-        <v>26276.79</v>
-      </c>
-      <c r="DP36">
-        <v>6299826.7599999998</v>
-      </c>
-      <c r="DQ36">
-        <v>26276.79</v>
-      </c>
-      <c r="DR36">
-        <v>6299826.7599999998</v>
-      </c>
-      <c r="DW36">
-        <v>929.22</v>
-      </c>
-      <c r="DX36">
-        <v>26298.720000000001</v>
-      </c>
-      <c r="DY36">
-        <v>2</v>
-      </c>
-      <c r="DZ36">
-        <v>2</v>
-      </c>
-      <c r="EA36">
-        <v>929.22</v>
-      </c>
-      <c r="EB36">
-        <v>26298.720000000001</v>
-      </c>
-      <c r="EG36">
-        <v>2</v>
-      </c>
-      <c r="EH36">
-        <v>2</v>
-      </c>
-      <c r="EJ36">
-        <v>929.22</v>
-      </c>
-      <c r="EK36">
-        <v>26298.720000000001</v>
-      </c>
-      <c r="EL36" t="s">
-        <v>174</v>
-      </c>
-      <c r="EM36" s="1"/>
-    </row>
-    <row r="37" spans="1:143" x14ac:dyDescent="0.25">
-      <c r="D37">
-        <v>7003</v>
-      </c>
-      <c r="F37" t="s">
-        <v>243</v>
-      </c>
-      <c r="H37" s="1"/>
-      <c r="I37" s="1"/>
-      <c r="S37">
-        <v>14008840</v>
-      </c>
-      <c r="AM37" s="1"/>
-      <c r="BF37" s="1"/>
-      <c r="CB37" s="1"/>
-      <c r="CC37" s="1"/>
-      <c r="CO37" s="1"/>
-      <c r="CP37" s="1"/>
-      <c r="CW37">
-        <v>99649294194</v>
-      </c>
-      <c r="CX37">
-        <v>99649294194</v>
-      </c>
-      <c r="DO37">
-        <v>41211221112</v>
-      </c>
-      <c r="DP37">
-        <v>41211221112</v>
-      </c>
-      <c r="DQ37">
-        <v>69222669996</v>
-      </c>
-      <c r="DR37">
-        <v>69222669996</v>
-      </c>
-      <c r="DS37">
-        <v>196929027</v>
-      </c>
-      <c r="DT37">
-        <v>196929027</v>
-      </c>
-      <c r="DU37">
-        <v>2161.91</v>
-      </c>
-      <c r="DV37">
-        <v>2161.91</v>
-      </c>
-      <c r="DW37">
-        <v>11920144926</v>
-      </c>
-      <c r="DX37">
-        <v>11920144926</v>
-      </c>
-      <c r="DY37">
-        <v>0</v>
-      </c>
-      <c r="DZ37">
-        <v>0</v>
-      </c>
-      <c r="EA37">
-        <v>11920144926</v>
-      </c>
-      <c r="EB37">
-        <v>11920144926</v>
-      </c>
-      <c r="EC37">
-        <v>1102922205</v>
-      </c>
-      <c r="ED37">
-        <v>1102922205</v>
-      </c>
-      <c r="EE37">
-        <v>162299941.19999999</v>
-      </c>
-      <c r="EF37">
-        <v>162299941.19999999</v>
-      </c>
-      <c r="EG37">
-        <v>1929622297</v>
-      </c>
-      <c r="EH37">
-        <v>1929622297</v>
-      </c>
-      <c r="EJ37">
-        <v>9999422223</v>
-      </c>
-      <c r="EK37">
-        <v>9999422223</v>
-      </c>
-      <c r="EM37" s="1"/>
-    </row>
-    <row r="38" spans="1:143" x14ac:dyDescent="0.25">
-      <c r="D38">
-        <v>7003</v>
-      </c>
-      <c r="F38" t="s">
-        <v>244</v>
-      </c>
-      <c r="H38" s="1"/>
-      <c r="I38" s="1"/>
-      <c r="S38">
-        <v>14008840</v>
-      </c>
-      <c r="AM38" s="1"/>
-      <c r="BF38" s="1"/>
-      <c r="CB38" s="1"/>
-      <c r="CC38" s="1"/>
-      <c r="CO38" s="1"/>
-      <c r="CP38" s="1"/>
-      <c r="CW38">
-        <v>196414963</v>
-      </c>
-      <c r="CX38">
-        <v>2626291200</v>
-      </c>
-      <c r="DO38">
-        <v>10409999.210000001</v>
-      </c>
-      <c r="DP38">
-        <v>6911299130</v>
-      </c>
-      <c r="DQ38">
-        <v>40246419.020000003</v>
-      </c>
-      <c r="DR38">
-        <v>1961909125</v>
-      </c>
-      <c r="DS38">
-        <v>4964246.6900000004</v>
-      </c>
-      <c r="DT38">
-        <v>4964246.6900000004</v>
-      </c>
-      <c r="DW38">
-        <v>22262666.960000001</v>
-      </c>
-      <c r="DX38">
-        <v>1622242901</v>
-      </c>
-      <c r="DY38">
-        <v>0</v>
-      </c>
-      <c r="DZ38">
-        <v>0</v>
-      </c>
-      <c r="EA38">
-        <v>22262666.960000001</v>
-      </c>
-      <c r="EB38">
-        <v>1622242901</v>
-      </c>
-      <c r="EC38">
-        <v>6642212.96</v>
-      </c>
-      <c r="ED38">
-        <v>126226091.3</v>
-      </c>
-      <c r="EE38">
-        <v>1912.96</v>
-      </c>
-      <c r="EF38">
-        <v>96162.04</v>
-      </c>
-      <c r="EG38">
-        <v>6644220.4900000002</v>
-      </c>
-      <c r="EH38">
-        <v>126119929.7</v>
-      </c>
-      <c r="EJ38">
-        <v>26912166.02</v>
-      </c>
-      <c r="EK38">
-        <v>1190422929</v>
-      </c>
-      <c r="EM38" s="1"/>
-    </row>
-    <row r="39" spans="1:143" x14ac:dyDescent="0.25">
-      <c r="D39">
-        <v>7003</v>
-      </c>
-      <c r="F39" t="s">
-        <v>232</v>
-      </c>
-      <c r="H39" s="1"/>
-      <c r="I39" s="1"/>
-      <c r="S39">
-        <v>14008840</v>
-      </c>
-      <c r="AM39" s="1"/>
-      <c r="BF39" s="1"/>
-      <c r="CB39" s="1"/>
-      <c r="CC39" s="1"/>
-      <c r="CO39" s="1"/>
-      <c r="CP39" s="1"/>
-      <c r="CW39">
-        <v>641296994.29999995</v>
-      </c>
-      <c r="CX39">
-        <v>14699610997</v>
-      </c>
-      <c r="DO39">
-        <v>119160966.09999999</v>
-      </c>
-      <c r="DP39">
-        <v>2122900611</v>
-      </c>
-      <c r="DQ39">
-        <v>161196296</v>
-      </c>
-      <c r="DR39">
-        <v>6216142044</v>
-      </c>
-      <c r="DS39">
-        <v>9441440</v>
-      </c>
-      <c r="DT39">
-        <v>6201169.2000000002</v>
-      </c>
-      <c r="DW39">
-        <v>99492692.189999998</v>
-      </c>
-      <c r="DX39">
-        <v>4116649923</v>
-      </c>
-      <c r="DY39">
-        <v>0</v>
-      </c>
-      <c r="DZ39">
-        <v>0</v>
-      </c>
-      <c r="EA39">
-        <v>99492692.189999998</v>
-      </c>
-      <c r="EB39">
-        <v>4116649923</v>
-      </c>
-      <c r="EC39">
-        <v>64696442.289999999</v>
-      </c>
-      <c r="ED39">
-        <v>1446622123</v>
-      </c>
-      <c r="EE39">
-        <v>9292194.9000000004</v>
-      </c>
-      <c r="EF39">
-        <v>244099942.5</v>
-      </c>
-      <c r="EG39">
-        <v>40194292.189999998</v>
-      </c>
-      <c r="EH39">
-        <v>1612611665</v>
-      </c>
-      <c r="EJ39">
-        <v>99266699</v>
-      </c>
-      <c r="EK39">
-        <v>2491961612</v>
-      </c>
-      <c r="EM39" s="1"/>
-    </row>
-    <row r="40" spans="1:143" x14ac:dyDescent="0.25">
-      <c r="D40">
-        <v>7003</v>
-      </c>
-      <c r="F40" t="s">
-        <v>245</v>
-      </c>
-      <c r="H40" s="1"/>
-      <c r="I40" s="1"/>
-      <c r="S40">
-        <v>14008840</v>
-      </c>
-      <c r="AM40" s="1"/>
-      <c r="BF40" s="1"/>
-      <c r="CB40" s="1"/>
-      <c r="CC40" s="1"/>
-      <c r="CO40" s="1"/>
-      <c r="CP40" s="1"/>
-      <c r="CX40">
-        <v>22621264602</v>
-      </c>
-      <c r="DP40">
-        <v>96029412030</v>
-      </c>
-      <c r="DR40">
-        <v>44426012423</v>
-      </c>
-      <c r="DT40">
-        <v>201962999</v>
-      </c>
-      <c r="DV40">
-        <v>2161.91</v>
-      </c>
-      <c r="DX40">
-        <v>12014242405</v>
-      </c>
-      <c r="DZ40">
-        <v>0</v>
-      </c>
-      <c r="EB40">
-        <v>12014242405</v>
-      </c>
-      <c r="ED40">
-        <v>6422912119</v>
-      </c>
-      <c r="EF40">
-        <v>411999991.69999999</v>
-      </c>
-      <c r="EH40">
-        <v>6169126146</v>
-      </c>
-      <c r="EK40">
-        <v>16244161960</v>
-      </c>
-      <c r="EM40" s="1"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>